<commit_message>
feat: update Sheet Riwayat Hukuman Disiplin
</commit_message>
<xml_diff>
--- a/public/template_excel/DATA PEGAWAI ASN.xlsx
+++ b/public/template_excel/DATA PEGAWAI ASN.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7755"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7755" firstSheet="7" activeTab="10"/>
   </bookViews>
   <sheets>
     <sheet name="Data Pegawai" sheetId="1" r:id="rId1"/>
@@ -79,7 +79,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="119">
   <si>
     <t>Golongan</t>
   </si>
@@ -252,9 +252,6 @@
     <t>Jenis Hukuman *</t>
   </si>
   <si>
-    <t>Tanggal Hukuman Disiplin *</t>
-  </si>
-  <si>
     <t>Nama Riwayat Hukuman Disiplin *</t>
   </si>
   <si>
@@ -433,6 +430,12 @@
   </si>
   <si>
     <t>Tanggal SK *</t>
+  </si>
+  <si>
+    <t>Tanggal Awal Hukuman Disiplin *</t>
+  </si>
+  <si>
+    <t>Tanggal Akhir Hukuman Disiplin *</t>
   </si>
 </sst>
 </file>
@@ -828,7 +831,7 @@
   <sheetData>
     <row r="1" spans="1:37" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>7</v>
@@ -837,61 +840,61 @@
         <v>8</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>1</v>
       </c>
       <c r="F1" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="G1" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="K1" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="L1" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="N1" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="O1" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="P1" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="Q1" s="2" t="s">
         <v>102</v>
-      </c>
-      <c r="M1" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="N1" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="O1" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="P1" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="Q1" s="2" t="s">
-        <v>103</v>
       </c>
       <c r="R1" s="2" t="s">
         <v>10</v>
       </c>
       <c r="S1" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="T1" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="U1" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="V1" s="2" t="s">
         <v>73</v>
-      </c>
-      <c r="V1" s="2" t="s">
-        <v>74</v>
       </c>
       <c r="W1" s="2" t="s">
         <v>12</v>
@@ -903,16 +906,16 @@
         <v>13</v>
       </c>
       <c r="Z1" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="AA1" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="AB1" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="AA1" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="AB1" s="2" t="s">
+      <c r="AC1" s="2" t="s">
         <v>76</v>
-      </c>
-      <c r="AC1" s="2" t="s">
-        <v>77</v>
       </c>
       <c r="AD1" s="2" t="s">
         <v>14</v>
@@ -933,10 +936,10 @@
         <v>19</v>
       </c>
       <c r="AJ1" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="AK1" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="2" spans="1:37" x14ac:dyDescent="0.25">
@@ -972,22 +975,22 @@
   <sheetData>
     <row r="1" spans="1:7" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>91</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>92</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>55</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>43</v>
@@ -1000,7 +1003,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="35.42578125" style="1" bestFit="1" customWidth="1"/>
@@ -1012,20 +1015,21 @@
     <col min="7" max="7" width="26.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="25.7109375" style="1" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="30" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="28.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="12" width="26.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="13" max="16384" width="9.140625" style="1"/>
+    <col min="10" max="10" width="34.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="34.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="13" width="26.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="14" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="C1" s="2" t="s">
         <v>59</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>60</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>55</v>
@@ -1046,19 +1050,22 @@
         <v>45</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>57</v>
+        <v>117</v>
       </c>
       <c r="K1" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="L1" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="M1" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="N1" s="2" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="2" spans="1:13" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:14" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" s="1"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -1107,25 +1114,25 @@
         <v>55</v>
       </c>
       <c r="B1" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="C1" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="C1" s="3" t="s">
-        <v>82</v>
-      </c>
       <c r="D1" s="3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G1" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="H1" s="3" t="s">
         <v>63</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>64</v>
       </c>
       <c r="I1" s="3" t="s">
         <v>49</v>
@@ -1134,10 +1141,10 @@
         <v>50</v>
       </c>
       <c r="K1" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="L1" s="3" t="s">
         <v>83</v>
-      </c>
-      <c r="L1" s="3" t="s">
-        <v>84</v>
       </c>
       <c r="M1" s="3" t="s">
         <v>51</v>
@@ -1146,7 +1153,7 @@
         <v>52</v>
       </c>
       <c r="O1" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="P1" s="3" t="s">
         <v>16</v>
@@ -1181,19 +1188,19 @@
         <v>55</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="D1" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>109</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>110</v>
       </c>
     </row>
   </sheetData>
@@ -1216,7 +1223,7 @@
         <v>55</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
   </sheetData>
@@ -1242,10 +1249,10 @@
         <v>55</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>38</v>
@@ -1274,10 +1281,10 @@
         <v>55</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>38</v>
@@ -1306,10 +1313,10 @@
         <v>55</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>38</v>
@@ -1341,10 +1348,10 @@
         <v>55</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>2</v>
@@ -1353,10 +1360,10 @@
         <v>3</v>
       </c>
       <c r="F1" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="G1" s="2" t="s">
         <v>79</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>80</v>
       </c>
       <c r="H1" s="2" t="s">
         <v>20</v>
@@ -1396,19 +1403,19 @@
   <sheetData>
     <row r="1" spans="1:18" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>59</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>60</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>55</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F1" s="2" t="s">
         <v>21</v>
@@ -1420,7 +1427,7 @@
         <v>23</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="J1" s="2" t="s">
         <v>24</v>
@@ -1477,22 +1484,22 @@
   <sheetData>
     <row r="1" spans="1:12" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>59</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>60</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>55</v>
       </c>
       <c r="E1" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="F1" s="2" t="s">
         <v>69</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>70</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>4</v>
@@ -1537,22 +1544,22 @@
   <sheetData>
     <row r="1" spans="1:9" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>112</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>113</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>36</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>37</v>
@@ -1586,22 +1593,22 @@
   <sheetData>
     <row r="1" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>112</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>113</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>36</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>37</v>
@@ -1634,19 +1641,19 @@
   <sheetData>
     <row r="1" spans="1:7" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="B1" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>113</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>114</v>
       </c>
       <c r="F1" s="2" t="s">
         <v>37</v>
@@ -1681,25 +1688,25 @@
   <sheetData>
     <row r="1" spans="1:11" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>59</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>60</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>39</v>
       </c>
       <c r="E1" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="F1" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="F1" s="2" t="s">
-        <v>117</v>
-      </c>
       <c r="G1" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="H1" s="2" t="s">
         <v>40</v>
@@ -1738,16 +1745,16 @@
   <sheetData>
     <row r="1" spans="1:9" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>94</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>95</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>11</v>
@@ -1756,13 +1763,13 @@
         <v>55</v>
       </c>
       <c r="G1" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="H1" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>97</v>
-      </c>
-      <c r="I1" s="2" t="s">
-        <v>98</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: import excel add column nama and add comment on column with option
</commit_message>
<xml_diff>
--- a/public/template_excel/DATA PEGAWAI ASN.xlsx
+++ b/public/template_excel/DATA PEGAWAI ASN.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7755" firstSheet="7" activeTab="10"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7755" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Data Pegawai" sheetId="1" r:id="rId1"/>
@@ -45,6 +45,115 @@
     <author>Windows User</author>
   </authors>
   <commentList>
+    <comment ref="H1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Agama</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+- Islam
+- Kristen
+- Katolik
+- Hindu
+- Budha
+- Konghucu</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="I1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Jenis Kelamin</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+- Perempuan
+- Laki-laki</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="J1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Status Perkawinan</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+- Belum Menikah
+- Menikah
+- Cerai
+- Janda
+- Duda</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="K1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Jenis Pegawai</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+TNI/POLRI
+SIPIL
+ORGANIK
+PPPK</t>
+        </r>
+      </text>
+    </comment>
     <comment ref="M1" authorId="0" shapeId="0">
       <text>
         <r>
@@ -55,7 +164,8 @@
             <rFont val="Tahoma"/>
             <charset val="1"/>
           </rPr>
-          <t>Windows User:</t>
+          <t xml:space="preserve">Jabatan
+</t>
         </r>
         <r>
           <rPr>
@@ -74,12 +184,1478 @@
         </r>
       </text>
     </comment>
+    <comment ref="O1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Golongan
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Pembina Utama
+Pembina Utama Madya
+Pembina Utama Muda
+Pembina Tingkat I
+Pembina
+Penata Tingkat I
+Penata
+Penata Muda Tingkat I
+Penata Muda
+Pengatur Tingkat I
+Pengatur
+Pengatur Muda Tingkat I
+Pengatur Muda
+Juru Tingkat I
+Juru
+Juru Muda Tingkat I
+Juru Muda
+Golongan XVII
+Golongan XVI
+Golongan XV
+Golongan XIV
+Golongan XIII
+Golongan XII
+Golongan XI
+Golongan X
+Golongan IX
+Golongan VIII
+Golongan VII
+Golongan VI
+Golongan V
+Golongan IV
+Golongan III
+Golongan II
+Golongan </t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="Q1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Eselon
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Eselon I
+Eselon II
+Eselon III
+Eselon IV
+Ahli Utama
+Ahli Madya
+Ahli Muda
+Ahli Pertama
+Pelaksana
+Penyelia
+Mahir
+Terampil
+Pemula</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="S1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Instansi Induk</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Kementerian Sekretariat Negara
+Kementerian Perindustrian dan Perdagangan
+Kementerian Perdagangan
+Kementerian Riset, Teknologi dan Pendidikan Tinggi
+Kementerian Luar Negeri
+Kementerian Koordinator Bidang Pembangunan Manusia dan Kebudayaan
+Kementerian Keuangan
+Kementerian Hukum dan HAM
+Kementerian Dalam Negeri
+Kementerian PPN/ Bappenas
+Kementerian Sosial
+Departemen Pekerjaan Umum
+Departemen Luar Negeri
+Departemen Dalam Negeri
+Badan Pengawas Keuangan dan Pembangunan (BPKP)
+Lembaga Ilmu Pengetahuan Indonesia (LIPI)
+Perpustakaan Nasional
+Lembaga Administrasi Negara (LAN)
+Badan Kepegawaian Negara (BKN)
+Pemerintah Kota Surabaya Provinsi Jawa Timur
+Sekretariat Militer Presiden
+Markas Besar TNI
+Pasukan Pengamanan Presiden (Paspampres)
+Pemerintah Provinsi DKI Jakarta
+Markas Besar POLRI
+Kementerian Pendidikan dan Kebudayaan
+Badan Siber dan Sandi Negara</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="T1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Tingkat Pendidikan Terakhir</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+- SD/Sederajat
+- SLTP/Sederajat
+- SLTA/Sederajat
+- Diploma I/II
+- Akademik/D3/S.Muda
+- Diploma IV/Strata I
+- Strata II
+- Strata III</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="Z1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Status Pegawai</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+- Aktif
+- Pensiun
+- Berhenti
+- Meninggal
+- Alih Status
+- Aktif Perbantuan Setneg
+- CLTN
+- TBLN
+- Non Aktif</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AC1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Komplek</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+- Luar Komplek
+- Cempaka Putih (Komplek Setneg Cempaka Putih, Jakarta Pusat)
+- Sunter (Komplek Setneg Sunter Agung, Tanjung Priok, Jakarta Utara)
+- Cidodol (Komplek Setneg Cidodol, Grogol Selatan, Keb.Lama, Jakarta Selatan)
+- Ciledug (Komplek Setneg, Pd. Kacang Barat, Pd. Aren, Tangerang)
+- Suradita (Komplek Setneg, Perumahan Suradita, Cisauk, Tangerang)
+- Karawaci (Komplek Setneg, Bencongan Indah, Kelapa Dua, Tangerang)
+- Plumpang (Komplek Setneg, Tugu Utara, Koja, Jakarta Utara)
+- Jonggol (Komplek Setwapres, Perum.Griya Merselina, Desa Suka Galih, Kec. Jonggol, Kab. Bogor)
+- Cipondoh (Komplek Setneg, Panunggangan Utara, Kec. Pinang, Tangerang)</t>
+        </r>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
 
+<file path=xl/comments10.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Windows User</author>
+  </authors>
+  <commentList>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Bulan</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+- Januari
+- Februari
+- Maret
+- April
+- Mei
+- Juni
+- Juli
+- Agustus
+- September
+- Oktober
+- November
+- Desember</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="H1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Keterangan</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+- Kurang
+- Sedang
+- Cukup
+- Baik
+- Sangat Baik</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments11.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Windows User</author>
+  </authors>
+  <commentList>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Bulan</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+- Januari
+- Februari
+- Maret
+- April
+- Mei
+- Juni
+- Juli
+- Agustus
+- September
+- Oktober
+- November
+- Desember</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="H1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Jenis Hukuman</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Teguran Lisan
+Teguran Tertulis
+Pernyataan Tidak Puas Secara Tertulis
+Penundaan Kenaikan Gaji Berkala Selama 1 (Satu) Tahun
+Penundaan Kenaikan Pangkat Selama 1 (Satu) Tahun
+Penurunan Pangkat Setingkat Lebih Rendah Selama 1 (Satu) Tahun
+Penurunan Pangkat Setingkat Lebih Rendah Selama 3 (Tiga) Tahun
+Pemindahan Dalam Rangka Penurunan Jabatan Setingkat Lebih Rendah
+Pembebasan Dari Jabatan
+Pemberhentian Dengan Hormat Tidak Atas Permintaan Sendiri Sebagai PNS
+Pemberhentian Tidak Dengan Hormat Sebagai PNS</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments12.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Windows User</author>
+  </authors>
+  <commentList>
+    <comment ref="F1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Jenis Kelamin</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+- Laki-laki
+- Perempuan</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">Agama
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>- Islam
+- Kristen
+- Katolik
+- Hindu
+- Budha
+- Konghucu</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="L1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Hubungan Keluarga</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+- Kepala Keluarga
+- Suami
+- Istri
+- Anak
+- Menantu
+- Cucu
+- Orang Tua
+- Mertua
+- Famili Lainnya
+- Pembantu
+- Lainnya</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="M1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Pendidikan</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+- Tidak/Belum Sekolah
+- Belum Tamat SD/Sederajat
+- Tamat SD/Sederajat
+- SLTP/Sederajat
+- SLTA/Sederajat
+- Diploma I/II
+- Akademi/diploma III/Sarjana Muda
+- Diploma IV/Strata I
+- Strata II
+- Strata III</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="P1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Status Perkawinan</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+- Belum Menikah
+- Menikah
+- Cerai Hidup
+- Cerai Mati</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments13.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Windows User</author>
+  </authors>
+  <commentList>
+    <comment ref="E1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Jenis Cuti</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+- Cuti Diluar Tanggungan Negara
+- Cuti Sakit
+- Cuti Besar
+- Cuti Bersalin
+- Cuti Belajar Luar Negeri
+- Cuti Tahunan Luar Negeri</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments14.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Windows User</author>
+  </authors>
+  <commentList>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Hasil</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+- Kurang Memenuhi Syarat
+- Masih Memenuhi Syarat
+- Memenuhi Syarat</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments15.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Windows User</author>
+  </authors>
+  <commentList>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Windows User:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+- Lulus
+- Tidak Lulus</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments16.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Windows User</author>
+  </authors>
+  <commentList>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Windows User:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+- Kotak 1
+- Kotak 2
+- Kotak 3
+- Kotak 4
+- Kotak 5
+- Kotak 6
+- Kotak 7
+- Kotak 8
+- Kotak 9</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Windows User</author>
+  </authors>
+  <commentList>
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Tingkat</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+- SD/Sederajat
+- SLTP/Sederajat
+- SLTA/Sederajat
+- Diploma I/II
+- Akademik/D3/S.Muda
+- Diploma IV/Strata I
+- Strata II
+- Strata III</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Status</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+- Lulus
+- DO
+- Aktif
+- Non-aktif
+- Mengundurkan Diri</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments3.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Windows User</author>
+  </authors>
+  <commentList>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Bulan</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+- Januari
+- Februari
+- Maret
+- April
+- Mei
+- Juni
+- Juli
+- Agustus
+- September
+- Oktober
+- November
+- Desember</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Rumpun</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+- Pengelolaan Sumber Daya Manusia 
+- Kelembagaan dan Tata Laksana
+- Pengembangan Kompetensi 
+- Bantuan Hukum
+- Perencanaan Program dan Anggaran
+- Akuntabilitas Kinerja
+- Keuangan
+- Audit Internal
+- Tata Usaha
+- Arsip
+- Perpustakaan
+- Perancangan Grafis
+- Pengelolaan Bangunan
+- Pengelolaan Kendaraan serta Perlengkapan dan Peralatan
+- Kerumahtanggaan/Tata Gerha
+- Pengamanan Dalam
+- Pelayanan Medis
+- Sistem Informasi
+- Infrastruktur
+- Pengelolaan Informasi Publik
+- Peliputan dan Dokumentasi
+- Protokol VVIP dan VIP
+- Ajudan VVIP dan VIP
+- Pengelolaan Benda Seni dan Budaya
+- Pengamanan VIP dan VVIP
+- Analisis Kebijakan
+- Analisis Pengaduan Masyarakat
+- Analisis Hukum dan Perundang-undangan
+- Kerja Sama Teknik dan Tenaga Asing
+- Penetapan Pengangkatan/Pemberhentian/ Pensiun/Cuti bagi Pejabat Negara/Pejabat Pemerintah/Perwira TNI/POLRI
+- Penetapan Gelar, Tanda Jasa, dan Tanda Kehormatan
+- Perjalanan Dinas Luar Negeri</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="H1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Jenjang Jabatan</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+- Eselon I
+- Eselon II
+- Eselon III
+- Fungsional
+- Pelaksana
+- Staf</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="I1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Keterangan Jabatan</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+- Promosi
+- Mutasi
+- Inpassing
+- Konversi</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments4.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Windows User</author>
+  </authors>
+  <commentList>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Bulan</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+- Januari
+- Februari
+- Maret
+- April
+- Mei
+- Juni
+- Juli
+- Agustus
+- September
+- Oktober
+- November
+- Desember</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Golongan</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Pembina Utama
+Pembina Utama Madya
+Pembina Utama Muda
+Pembina Tingkat I
+Pembina
+Penata Tingkat I
+Penata
+Penata Muda Tingkat I
+Penata Muda
+Pengatur Tingkat I
+Pengatur
+Pengatur Muda Tingkat I
+Pengatur Muda
+Juru Tingkat I
+Juru
+Juru Muda Tingkat I
+Juru Muda
+Golongan XVII
+Golongan XVI
+Golongan XV
+Golongan XIV
+Golongan XIII
+Golongan XII
+Golongan XI
+Golongan X
+Golongan IX
+Golongan VIII
+Golongan VII
+Golongan VI
+Golongan V
+Golongan IV
+Golongan III
+Golongan II
+Golongan I</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="I1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Jenis SK Golongan</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Keputusan Presiden
+Keputusan Menteri Sekretaris Negara
+Keputusan Sekretaris Negara
+Keputusan Sekretaris Wakil Presiden
+Keputusan Menteri Perencanaan Pembangunan Nasional Bappenas
+Keputusan Menteri PUPR
+Keputusan Kepala Staf Angkatan Laut
+Keputusan Kepala Staf Angkatan Darat
+Surat Telegram Kapolri
+Keputusan Kepala Badan Siber dan Sandi Negara
+Keputusan Menteri Koperasi dan Usaha Kecil dan Menengah
+Keputusan Deputi Bidang Sumber Daya Manusia
+Keputusan Menteri Hukum dan HAM
+Keputusan Kepala Staf Angkatan Udara
+Keputusan Menteri PPN
+Keputusan Koordinator Bidang Pembangunan Manusia dan Kebudayaan Republik Indonesia</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="M1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Status Golongan</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+- Aktif
+- Tidak Aktif</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments5.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Windows User</author>
+  </authors>
+  <commentList>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Bulan</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+- Januari
+- Februari
+- Maret
+- April
+- Mei
+- Juni
+- Juli
+- Agustus
+- September
+- Oktober
+- November
+- Desember</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments6.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Windows User</author>
+  </authors>
+  <commentList>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Bulan</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+- Januari
+- Februari
+- Maret
+- April
+- Mei
+- Juni
+- Juli
+- Agustus
+- September
+- Oktober
+- November
+- Desember</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments7.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Windows User</author>
+  </authors>
+  <commentList>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Bulan</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+- Januari
+- Februari
+- Maret
+- April
+- Mei
+- Juni
+- Juli
+- Agustus
+- September
+- Oktober
+- November
+- Desember</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments8.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Windows User</author>
+  </authors>
+  <commentList>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Bulan</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+- Januari
+- Februari
+- Maret
+- April
+- Mei
+- Juni
+- Juli
+- Agustus
+- September
+- Oktober
+- November
+- Desember</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Jenis SK</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Keputusan Presiden
+Keputusan Menteri Sekretaris Negara
+Keputusan Sekretaris Negara
+Keputusan Sekretaris Wakil Presiden
+Keputusan Menteri Perencanaan Pembangunan Nasional Bappenas
+Keputusan Menteri PUPR
+Keputusan Kepala Staf Angkatan Laut
+Keputusan Kepala Staf Angkatan Darat
+Surat Telegram Kapolri
+Keputusan Kepala Badan Siber dan Sandi Negara
+Keputusan Menteri Koperasi dan Usaha Kecil dan Menengah
+Keputusan Deputi Bidang Sumber Daya Manusia
+Keputusan Menteri Hukum dan HAM
+Keputusan Kepala Staf Angkatan Udara
+Keputusan Menteri PPN
+Keputusan Koordinator Bidang Pembangunan Manusia dan Kebudayaan Republik Indonesia</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments9.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Windows User</author>
+  </authors>
+  <commentList>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Bulan</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+- Januari
+- Februari
+- Maret
+- April
+- Mei
+- Juni
+- Juli
+- Agustus
+- September
+- Oktober
+- November
+- Desember</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Periode Penilaian</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+- Q1
+- Q2
+- Q3
+- Q4
+- Tahunan</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="H1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Rating Perilaku Kerja</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+- Diatas Ekspektasi
+- Sesuai Ekspektasi
+- Dibawah Ekspektasi</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="I1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Predikat Kinerja Pegawai</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+- Sangat Baik
+- Baik
+- Butuh Perbaikan
+- Kurang
+- Sangat Kurang</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="J1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Capaian Kinerja Organisasi</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+- Sangat Baik
+- Baik
+- Cukup</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="119">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="120">
   <si>
     <t>Golongan</t>
   </si>
@@ -436,13 +2012,16 @@
   </si>
   <si>
     <t>Tanggal Akhir Hukuman Disiplin *</t>
+  </si>
+  <si>
+    <t>Nama</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -478,6 +2057,19 @@
       <color indexed="81"/>
       <name val="Tahoma"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -959,8 +2551,8 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:H1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24.7109375" style="1" bestFit="1" customWidth="1"/>
@@ -968,12 +2560,13 @@
     <col min="3" max="3" width="32" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="18.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="24.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="21.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="18.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="16384" width="9.140625" style="1"/>
+    <col min="6" max="6" width="24.7109375" style="1" customWidth="1"/>
+    <col min="7" max="7" width="21.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>90</v>
       </c>
@@ -990,38 +2583,43 @@
         <v>55</v>
       </c>
       <c r="F1" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="G1" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>43</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:N2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="35.42578125" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="31.42578125" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="32" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="17.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="22.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="26.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="25.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="30" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="34.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="34.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="13" width="26.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="14" max="16384" width="9.140625" style="1"/>
+    <col min="5" max="5" width="17.28515625" style="1" customWidth="1"/>
+    <col min="6" max="6" width="22.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="26.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="25.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="30" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="34.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="34.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="13" max="14" width="26.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="15" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>57</v>
       </c>
@@ -1035,37 +2633,40 @@
         <v>55</v>
       </c>
       <c r="E1" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="F1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="K1" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="L1" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="M1" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="N1" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="N1" s="2" t="s">
+      <c r="O1" s="2" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="2" spans="1:14" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:15" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" s="1"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -1079,329 +2680,366 @@
       <c r="K2" s="1"/>
       <c r="L2" s="1"/>
       <c r="M2" s="1"/>
+      <c r="N2" s="1"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:R1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="22.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.42578125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="21" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="27" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="22.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="25" style="1" bestFit="1" customWidth="1"/>
+    <col min="14" max="15" width="24.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="21.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="13.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="14.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="19" max="16384" width="9.140625" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:18" s="3" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L1" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="M1" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="N1" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="O1" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="P1" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="Q1" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" s="3" t="s">
+        <v>53</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:G1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="22.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.42578125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="21.140625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="21.7109375" style="1" customWidth="1"/>
+    <col min="5" max="5" width="29.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.140625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="16.28515625" style="1" customWidth="1"/>
+    <col min="8" max="8" width="10.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="16384" width="9.140625" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>109</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:C1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="22.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.42578125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="23.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="16384" width="9.140625" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>84</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Q1"/>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:E1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="27" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="22.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="25" style="1" bestFit="1" customWidth="1"/>
-    <col min="13" max="14" width="24.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="21.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="13.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="14.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="18" max="16384" width="9.140625" style="1"/>
+    <col min="2" max="2" width="22.42578125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="10.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18" style="1" customWidth="1"/>
+    <col min="6" max="6" width="16.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" s="3" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="B1" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="J1" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="K1" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="L1" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="M1" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="N1" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="O1" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="P1" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="Q1" s="3" t="s">
-        <v>53</v>
+      <c r="B1" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="22.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.42578125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="10.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.28515625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="15.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="16384" width="9.140625" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="22.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.42578125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="10.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.28515625" style="1" customWidth="1"/>
+    <col min="6" max="6" width="16.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="16384" width="9.140625" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:I1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="22.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.42578125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="22.5703125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="19.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9" style="1" customWidth="1"/>
+    <col min="7" max="7" width="8.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="20.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="16384" width="9.140625" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>20</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="22.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.140625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="21.7109375" style="1" customWidth="1"/>
-    <col min="4" max="4" width="29.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.140625" style="1" customWidth="1"/>
-    <col min="6" max="6" width="16.28515625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="10.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="16384" width="9.140625" style="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:6" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>109</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="22.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="23.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="16384" width="9.140625" style="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:2" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>84</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="22.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18" style="1" customWidth="1"/>
-    <col min="5" max="5" width="16.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="16384" width="9.140625" style="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>38</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="22.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.28515625" style="1" customWidth="1"/>
-    <col min="4" max="4" width="15.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="16384" width="9.140625" style="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>38</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="22.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.28515625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="16.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="16384" width="9.140625" style="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>38</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="22.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.5703125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="19.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9" style="1" customWidth="1"/>
-    <col min="6" max="6" width="8.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="20.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="16384" width="9.140625" style="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:8" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>20</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:R1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:S1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="31.5703125" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="31.42578125" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="32" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="22.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="31.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="24.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="16.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="20.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="20" style="1" customWidth="1"/>
-    <col min="10" max="10" width="11.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="16.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="15.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="20" style="1" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="16.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="19" style="1" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="15.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="27.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="24.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="19" max="16384" width="9.140625" style="1"/>
+    <col min="5" max="5" width="22.42578125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="31.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="24.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="20.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="20" style="1" customWidth="1"/>
+    <col min="11" max="11" width="11.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="16.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="15.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="20" style="1" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="16.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="19" style="1" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="15.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="27.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="24.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="20" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:19" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>86</v>
       </c>
@@ -1415,74 +3053,79 @@
         <v>55</v>
       </c>
       <c r="E1" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="F1" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="K1" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="L1" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="M1" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="N1" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N1" s="2" t="s">
+      <c r="O1" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="O1" s="2" t="s">
+      <c r="P1" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="P1" s="2" t="s">
+      <c r="Q1" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="Q1" s="2" t="s">
+      <c r="R1" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="R1" s="2" t="s">
+      <c r="S1" s="2" t="s">
         <v>32</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:M1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="32.42578125" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="31.42578125" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="32" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="17.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="17.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="22" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="22.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="22" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="22.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="17.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="13" max="16384" width="9.140625" style="1"/>
+    <col min="5" max="5" width="17.28515625" style="1" customWidth="1"/>
+    <col min="6" max="6" width="18.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="22" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="22.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="22" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="22.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="17.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="14" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>89</v>
       </c>
@@ -1496,39 +3139,43 @@
         <v>55</v>
       </c>
       <c r="E1" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="F1" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="K1" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="L1" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="M1" s="2" t="s">
         <v>35</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:J1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26" style="1" bestFit="1" customWidth="1"/>
@@ -1542,7 +3189,7 @@
     <col min="10" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>111</v>
       </c>
@@ -1569,16 +3216,20 @@
       </c>
       <c r="I1" s="2" t="s">
         <v>55</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>119</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:J1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="53.7109375" style="1" bestFit="1" customWidth="1"/>
@@ -1591,7 +3242,7 @@
     <col min="10" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>111</v>
       </c>
@@ -1618,16 +3269,21 @@
       </c>
       <c r="I1" s="2" t="s">
         <v>55</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>119</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:H1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="54" style="1" customWidth="1"/>
@@ -1639,7 +3295,7 @@
     <col min="8" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>111</v>
       </c>
@@ -1660,16 +3316,20 @@
       </c>
       <c r="G1" s="2" t="s">
         <v>55</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>119</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:L1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.42578125" style="1" bestFit="1" customWidth="1"/>
@@ -1686,7 +3346,7 @@
     <col min="12" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>98</v>
       </c>
@@ -1719,16 +3379,20 @@
       </c>
       <c r="K1" s="2" t="s">
         <v>55</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>119</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:J1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.7109375" style="1" bestFit="1" customWidth="1"/>
@@ -1737,13 +3401,14 @@
     <col min="4" max="4" width="26" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="10.85546875" style="1" customWidth="1"/>
     <col min="6" max="6" width="17.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="23.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="27.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="29" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="16384" width="9.140625" style="1"/>
+    <col min="7" max="7" width="17.28515625" style="1" customWidth="1"/>
+    <col min="8" max="8" width="23.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="27.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="29" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>93</v>
       </c>
@@ -1763,16 +3428,20 @@
         <v>55</v>
       </c>
       <c r="G1" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="H1" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>97</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add nama komplek in import excel #2
</commit_message>
<xml_diff>
--- a/public/template_excel/DATA PEGAWAI ASN.xlsx
+++ b/public/template_excel/DATA PEGAWAI ASN.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7755" activeTab="2"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7755"/>
   </bookViews>
   <sheets>
     <sheet name="Data Pegawai" sheetId="1" r:id="rId1"/>
@@ -1655,7 +1655,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="121">
   <si>
     <t>Golongan</t>
   </si>
@@ -2015,6 +2015,9 @@
   </si>
   <si>
     <t>Nama</t>
+  </si>
+  <si>
+    <t>Nama Komplek</t>
   </si>
 </sst>
 </file>
@@ -2382,7 +2385,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AK5"/>
+  <dimension ref="A1:AL5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.42578125" style="1" bestFit="1" customWidth="1"/>
@@ -2411,17 +2414,18 @@
     <col min="26" max="26" width="23" style="1" bestFit="1" customWidth="1"/>
     <col min="27" max="28" width="17.28515625" style="1" bestFit="1" customWidth="1"/>
     <col min="29" max="29" width="58.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="67" style="1" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="20" style="1" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="7.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="15.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="19.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="35" max="36" width="25.28515625" style="1" customWidth="1"/>
-    <col min="37" max="37" width="73.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="38" max="16384" width="9.140625" style="1"/>
+    <col min="30" max="30" width="58.28515625" style="1" customWidth="1"/>
+    <col min="31" max="31" width="67" style="1" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="20" style="1" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="7.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="15.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="19.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="36" max="37" width="25.28515625" style="1" customWidth="1"/>
+    <col min="38" max="38" width="73.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="39" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:37" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:38" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>60</v>
       </c>
@@ -2510,39 +2514,42 @@
         <v>76</v>
       </c>
       <c r="AD1" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="AE1" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="AE1" s="2" t="s">
+      <c r="AF1" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="AF1" s="2" t="s">
+      <c r="AG1" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="AG1" s="2" t="s">
+      <c r="AH1" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="AH1" s="2" t="s">
+      <c r="AI1" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="AI1" s="2" t="s">
+      <c r="AJ1" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="AJ1" s="2" t="s">
+      <c r="AK1" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="AK1" s="2" t="s">
+      <c r="AL1" s="2" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="2" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="AI2" s="4"/>
+    <row r="2" spans="1:38" x14ac:dyDescent="0.25">
       <c r="AJ2" s="4"/>
+      <c r="AK2" s="4"/>
     </row>
-    <row r="3" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="AI3" s="4"/>
+    <row r="3" spans="1:38" x14ac:dyDescent="0.25">
       <c r="AJ3" s="4"/>
+      <c r="AK3" s="4"/>
     </row>
-    <row r="5" spans="1:37" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="5" spans="1:38" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
feat: import excel add Masa Kerja Keseluruhan & Masa Kerja Golongan input
</commit_message>
<xml_diff>
--- a/public/template_excel/DATA PEGAWAI ASN.xlsx
+++ b/public/template_excel/DATA PEGAWAI ASN.xlsx
@@ -154,7 +154,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="M1" authorId="0" shapeId="0">
+    <comment ref="N1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -184,7 +184,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="O1" authorId="0" shapeId="0">
+    <comment ref="P1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -242,7 +242,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="Q1" authorId="0" shapeId="0">
+    <comment ref="R1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -279,7 +279,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="S1" authorId="0" shapeId="0">
+    <comment ref="T1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -329,7 +329,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="T1" authorId="0" shapeId="0">
+    <comment ref="U1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -360,7 +360,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="Z1" authorId="0" shapeId="0">
+    <comment ref="AE1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -392,7 +392,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AC1" authorId="0" shapeId="0">
+    <comment ref="AH1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -1655,7 +1655,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="200" uniqueCount="126">
   <si>
     <t>Golongan</t>
   </si>
@@ -2018,6 +2018,21 @@
   </si>
   <si>
     <t>Nama Komplek</t>
+  </si>
+  <si>
+    <t>TMT PNS</t>
+  </si>
+  <si>
+    <t>Masa Kerja Keseluruhan Jumlah Tahun</t>
+  </si>
+  <si>
+    <t>Masa Kerja Keseluruhan Jumlah Bulan</t>
+  </si>
+  <si>
+    <t>Masa Kerja Golongan Jumlah Tahun</t>
+  </si>
+  <si>
+    <t>Masa Kerja Golongan Jumlah Bulan</t>
   </si>
 </sst>
 </file>
@@ -2385,7 +2400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AL5"/>
+  <dimension ref="A1:AQ5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.42578125" style="1" bestFit="1" customWidth="1"/>
@@ -2399,33 +2414,37 @@
     <col min="9" max="9" width="15.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="21.42578125" style="1" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="20.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="14" width="19.28515625" style="1" customWidth="1"/>
-    <col min="15" max="15" width="21.5703125" style="1" customWidth="1"/>
-    <col min="16" max="16" width="17.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="10.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="12.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="33.140625" style="1" customWidth="1"/>
-    <col min="20" max="20" width="30.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="29" style="1" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="15.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="11.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="10.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="17.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="23" style="1" bestFit="1" customWidth="1"/>
-    <col min="27" max="28" width="17.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="58.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="58.28515625" style="1" customWidth="1"/>
-    <col min="31" max="31" width="67" style="1" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="20" style="1" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="7.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="15.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="19.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="36" max="37" width="25.28515625" style="1" customWidth="1"/>
-    <col min="38" max="38" width="73.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="39" max="16384" width="9.140625" style="1"/>
+    <col min="12" max="15" width="19.28515625" style="1" customWidth="1"/>
+    <col min="16" max="16" width="21.5703125" style="1" customWidth="1"/>
+    <col min="17" max="17" width="17.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="10.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="12.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="33.140625" style="1" customWidth="1"/>
+    <col min="21" max="21" width="30.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="29" style="1" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="15.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="10.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="39.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="39" style="1" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="36.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="36.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="17.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="23" style="1" bestFit="1" customWidth="1"/>
+    <col min="32" max="33" width="17.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="58.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="58.28515625" style="1" customWidth="1"/>
+    <col min="36" max="36" width="67" style="1" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="20" style="1" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="7.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="15.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="19.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="41" max="42" width="25.28515625" style="1" customWidth="1"/>
+    <col min="43" max="43" width="73.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="44" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:38" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:43" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>60</v>
       </c>
@@ -2463,93 +2482,104 @@
         <v>101</v>
       </c>
       <c r="M1" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="N1" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="N1" s="2" t="s">
+      <c r="O1" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="O1" s="2" t="s">
+      <c r="P1" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="P1" s="2" t="s">
+      <c r="Q1" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="Q1" s="2" t="s">
+      <c r="R1" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="R1" s="2" t="s">
+      <c r="S1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="S1" s="2" t="s">
+      <c r="T1" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="T1" s="2" t="s">
+      <c r="U1" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="U1" s="2" t="s">
+      <c r="V1" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="V1" s="2" t="s">
+      <c r="W1" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="W1" s="2" t="s">
+      <c r="X1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="X1" s="2" t="s">
+      <c r="Y1" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="Y1" s="2" t="s">
+      <c r="Z1" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="AA1" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="AB1" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="AC1" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="AD1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="Z1" s="2" t="s">
+      <c r="AE1" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="AA1" s="2" t="s">
+      <c r="AF1" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="AB1" s="2" t="s">
+      <c r="AG1" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="AC1" s="2" t="s">
+      <c r="AH1" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="AD1" s="2" t="s">
+      <c r="AI1" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="AE1" s="2" t="s">
+      <c r="AJ1" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="AF1" s="2" t="s">
+      <c r="AK1" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="AG1" s="2" t="s">
+      <c r="AL1" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="AH1" s="2" t="s">
+      <c r="AM1" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="AI1" s="2" t="s">
+      <c r="AN1" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="AJ1" s="2" t="s">
+      <c r="AO1" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="AK1" s="2" t="s">
+      <c r="AP1" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="AL1" s="2" t="s">
+      <c r="AQ1" s="2" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="2" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="AJ2" s="4"/>
-      <c r="AK2" s="4"/>
+    <row r="3" spans="1:43" x14ac:dyDescent="0.25">
+      <c r="AO3" s="4"/>
+      <c r="AP3" s="4"/>
     </row>
-    <row r="3" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="AJ3" s="4"/>
-      <c r="AK3" s="4"/>
-    </row>
-    <row r="5" spans="1:38" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="5" spans="1:43" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
feat(Feat-B-005): Import Employees new mandatory field and field changes
</commit_message>
<xml_diff>
--- a/public/template_excel/DATA PEGAWAI ASN.xlsx
+++ b/public/template_excel/DATA PEGAWAI ASN.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7755"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7755" firstSheet="12" activeTab="16"/>
   </bookViews>
   <sheets>
     <sheet name="Data Pegawai" sheetId="1" r:id="rId1"/>
@@ -127,7 +127,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="K1" authorId="0" shapeId="0">
+    <comment ref="N1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -154,7 +154,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="N1" authorId="0" shapeId="0">
+    <comment ref="Q1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -184,7 +184,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="P1" authorId="0" shapeId="0">
+    <comment ref="S1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -242,7 +242,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="R1" authorId="0" shapeId="0">
+    <comment ref="U1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -279,7 +279,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="T1" authorId="0" shapeId="0">
+    <comment ref="W1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -329,7 +329,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="U1" authorId="0" shapeId="0">
+    <comment ref="X1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -360,7 +360,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AE1" authorId="0" shapeId="0">
+    <comment ref="AH1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -392,7 +392,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AH1" authorId="0" shapeId="0">
+    <comment ref="AK1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -998,61 +998,6 @@
 - Oktober
 - November
 - Desember</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="G1" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t>Rumpun</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t xml:space="preserve">
-- Pengelolaan Sumber Daya Manusia 
-- Kelembagaan dan Tata Laksana
-- Pengembangan Kompetensi 
-- Bantuan Hukum
-- Perencanaan Program dan Anggaran
-- Akuntabilitas Kinerja
-- Keuangan
-- Audit Internal
-- Tata Usaha
-- Arsip
-- Perpustakaan
-- Perancangan Grafis
-- Pengelolaan Bangunan
-- Pengelolaan Kendaraan serta Perlengkapan dan Peralatan
-- Kerumahtanggaan/Tata Gerha
-- Pengamanan Dalam
-- Pelayanan Medis
-- Sistem Informasi
-- Infrastruktur
-- Pengelolaan Informasi Publik
-- Peliputan dan Dokumentasi
-- Protokol VVIP dan VIP
-- Ajudan VVIP dan VIP
-- Pengelolaan Benda Seni dan Budaya
-- Pengamanan VIP dan VVIP
-- Analisis Kebijakan
-- Analisis Pengaduan Masyarakat
-- Analisis Hukum dan Perundang-undangan
-- Kerja Sama Teknik dan Tenaga Asing
-- Penetapan Pengangkatan/Pemberhentian/ Pensiun/Cuti bagi Pejabat Negara/Pejabat Pemerintah/Perwira TNI/POLRI
-- Penetapan Gelar, Tanda Jasa, dan Tanda Kehormatan
-- Perjalanan Dinas Luar Negeri</t>
         </r>
       </text>
     </comment>
@@ -1655,7 +1600,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="200" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="203" uniqueCount="130">
   <si>
     <t>Golongan</t>
   </si>
@@ -1858,36 +1803,18 @@
     <t>Status Perkawinan *</t>
   </si>
   <si>
-    <t>Jenis Pegawai *</t>
-  </si>
-  <si>
     <t>Golongan *</t>
   </si>
   <si>
     <t>TMT Golongan *</t>
   </si>
   <si>
-    <t>Instansi Induk *</t>
-  </si>
-  <si>
     <t>Tingkat *</t>
   </si>
   <si>
-    <t>Nama Sekolah/Universitas *</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tahun Lulus * </t>
-  </si>
-  <si>
-    <t>Status Pegawai *</t>
-  </si>
-  <si>
     <t>No NIK *</t>
   </si>
   <si>
-    <t>Komplek *</t>
-  </si>
-  <si>
     <t>Nama Sekolah *</t>
   </si>
   <si>
@@ -1954,24 +1881,12 @@
     <t>Nama Penghargaan *</t>
   </si>
   <si>
-    <t>Kontak Darurat (Nama, Nomor Handphone, Hubungan dengan pegawai) *</t>
-  </si>
-  <si>
-    <t>No KK *</t>
-  </si>
-  <si>
     <t>TMT CPNS *</t>
   </si>
   <si>
     <t>Eselon</t>
   </si>
   <si>
-    <t>Tingkat Pendidikan Terakhir*</t>
-  </si>
-  <si>
-    <t>Email Dinas</t>
-  </si>
-  <si>
     <t>Tanggal Awal Cuti *</t>
   </si>
   <si>
@@ -2017,12 +1932,36 @@
     <t>Nama</t>
   </si>
   <si>
-    <t>Nama Komplek</t>
-  </si>
-  <si>
     <t>TMT PNS</t>
   </si>
   <si>
+    <t>Status Perkawinan</t>
+  </si>
+  <si>
+    <t>Tanggal Perkawinan</t>
+  </si>
+  <si>
+    <t>Keterangan Perkawinan</t>
+  </si>
+  <si>
+    <t>Keterangan Lainnya</t>
+  </si>
+  <si>
+    <t>Jenis Pegawai</t>
+  </si>
+  <si>
+    <t>Instansi Induk</t>
+  </si>
+  <si>
+    <t>Tingkat Pendidikan Akhir*</t>
+  </si>
+  <si>
+    <t>Nama Sekolah/Universitas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tahun Lulus </t>
+  </si>
+  <si>
     <t>Masa Kerja Keseluruhan Jumlah Tahun</t>
   </si>
   <si>
@@ -2033,13 +1972,31 @@
   </si>
   <si>
     <t>Masa Kerja Golongan Jumlah Bulan</t>
+  </si>
+  <si>
+    <t>Status Pegawai</t>
+  </si>
+  <si>
+    <t>No KK</t>
+  </si>
+  <si>
+    <t>Komplek</t>
+  </si>
+  <si>
+    <t>Alamat Sesuai KTP</t>
+  </si>
+  <si>
+    <t>Email Dinas *</t>
+  </si>
+  <si>
+    <t>Kontak Darurat (Nama, Nomor Handphone, Hubungan dengan pegawai)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2051,14 +2008,6 @@
       <b/>
       <sz val="12"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -2107,21 +2056,18 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -2400,7 +2346,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AQ5"/>
+  <dimension ref="A1:AT3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.42578125" style="1" bestFit="1" customWidth="1"/>
@@ -2414,37 +2360,43 @@
     <col min="9" max="9" width="15.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="21.42578125" style="1" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="20.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="15" width="19.28515625" style="1" customWidth="1"/>
-    <col min="16" max="16" width="21.5703125" style="1" customWidth="1"/>
-    <col min="17" max="17" width="17.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="10.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="12.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="33.140625" style="1" customWidth="1"/>
-    <col min="21" max="21" width="30.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="29" style="1" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="15.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="10.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="39.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="39" style="1" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="36.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="36.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="17.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="23" style="1" bestFit="1" customWidth="1"/>
-    <col min="32" max="33" width="17.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="58.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="58.28515625" style="1" customWidth="1"/>
-    <col min="36" max="36" width="67" style="1" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="20" style="1" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="7.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="15.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="19.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="41" max="42" width="25.28515625" style="1" customWidth="1"/>
-    <col min="43" max="43" width="73.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="44" max="16384" width="9.140625" style="1"/>
+    <col min="12" max="12" width="24.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="20.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="19.28515625" style="1" customWidth="1"/>
+    <col min="15" max="15" width="21.5703125" style="1" customWidth="1"/>
+    <col min="16" max="16" width="17.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="84.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="17.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="33.140625" style="1" customWidth="1"/>
+    <col min="20" max="20" width="30.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="21" max="22" width="29" style="1" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="28.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="27.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="27.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="31.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="31.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="29" style="1" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="39.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="58.28515625" style="1" customWidth="1"/>
+    <col min="31" max="31" width="36.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="36.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="17.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="23" style="1" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="19.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="36" max="37" width="25.28515625" style="1" customWidth="1"/>
+    <col min="38" max="38" width="73.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="27.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="20" style="1" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="13.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="15.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="19.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="44" max="44" width="16.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="15.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="73.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="47" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:43" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:46" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>60</v>
       </c>
@@ -2473,113 +2425,118 @@
         <v>65</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>66</v>
+        <v>111</v>
       </c>
       <c r="K1" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="N1" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="O1" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="P1" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="Q1" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="R1" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="S1" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="L1" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="M1" s="2" t="s">
+      <c r="T1" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="U1" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="V1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="W1" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="X1" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="Y1" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="Z1" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="AA1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="AB1" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="AC1" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="AD1" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="N1" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="O1" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="P1" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="Q1" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="R1" s="2" t="s">
-        <v>102</v>
-      </c>
-      <c r="S1" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="T1" s="2" t="s">
+      <c r="AE1" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="AF1" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="AG1" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="AH1" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="AI1" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="AJ1" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="U1" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="V1" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="W1" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="X1" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="Y1" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="Z1" s="2" t="s">
-        <v>122</v>
-      </c>
-      <c r="AA1" s="2" t="s">
-        <v>123</v>
-      </c>
-      <c r="AB1" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="AC1" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="AD1" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="AE1" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="AF1" s="2" t="s">
-        <v>100</v>
-      </c>
-      <c r="AG1" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="AH1" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="AI1" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="AJ1" s="2" t="s">
+      <c r="AK1" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="AL1" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="AK1" s="2" t="s">
+      <c r="AM1" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="AN1" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="AL1" s="2" t="s">
+      <c r="AO1" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="AM1" s="2" t="s">
+      <c r="AP1" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="AN1" s="2" t="s">
+      <c r="AQ1" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="AO1" s="2" t="s">
+      <c r="AR1" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="AP1" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="AQ1" s="2" t="s">
-        <v>99</v>
+      <c r="AS1" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="AT1" s="2" t="s">
+        <v>129</v>
       </c>
     </row>
-    <row r="3" spans="1:43" x14ac:dyDescent="0.25">
-      <c r="AO3" s="4"/>
-      <c r="AP3" s="4"/>
-    </row>
-    <row r="5" spans="1:43" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="3" spans="1:46" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -2605,7 +2562,7 @@
   <sheetData>
     <row r="1" spans="1:8" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>58</v>
@@ -2614,16 +2571,16 @@
         <v>59</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>55</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>119</v>
+        <v>109</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="H1" s="2" t="s">
         <v>43</v>
@@ -2637,7 +2594,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="35.42578125" style="1" bestFit="1" customWidth="1"/>
@@ -2670,7 +2627,7 @@
         <v>55</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>119</v>
+        <v>109</v>
       </c>
       <c r="F1" s="2" t="s">
         <v>0</v>
@@ -2688,10 +2645,10 @@
         <v>45</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>117</v>
+        <v>107</v>
       </c>
       <c r="L1" s="2" t="s">
-        <v>118</v>
+        <v>108</v>
       </c>
       <c r="M1" s="2" t="s">
         <v>46</v>
@@ -2702,22 +2659,6 @@
       <c r="O1" s="2" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="2" spans="1:15" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="1"/>
-      <c r="B2" s="1"/>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
-      <c r="G2" s="1"/>
-      <c r="H2" s="1"/>
-      <c r="I2" s="1"/>
-      <c r="J2" s="1"/>
-      <c r="K2" s="1"/>
-      <c r="L2" s="1"/>
-      <c r="M2" s="1"/>
-      <c r="N2" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2755,16 +2696,16 @@
         <v>55</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>119</v>
+        <v>109</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="F1" s="3" t="s">
         <v>65</v>
@@ -2785,10 +2726,10 @@
         <v>50</v>
       </c>
       <c r="L1" s="3" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="M1" s="3" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="N1" s="3" t="s">
         <v>51</v>
@@ -2834,22 +2775,22 @@
         <v>55</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>119</v>
+        <v>109</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>105</v>
+        <v>95</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>106</v>
+        <v>96</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>107</v>
+        <v>97</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>108</v>
+        <v>98</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>109</v>
+        <v>99</v>
       </c>
     </row>
   </sheetData>
@@ -2874,10 +2815,10 @@
         <v>55</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>119</v>
+        <v>109</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
     </row>
   </sheetData>
@@ -2904,13 +2845,13 @@
         <v>55</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>119</v>
+        <v>109</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>38</v>
@@ -2941,13 +2882,13 @@
         <v>55</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>119</v>
+        <v>109</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>38</v>
@@ -2978,13 +2919,13 @@
         <v>55</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>119</v>
+        <v>109</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>38</v>
@@ -3018,13 +2959,13 @@
         <v>55</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>119</v>
+        <v>109</v>
       </c>
       <c r="C1" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>71</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>77</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>2</v>
@@ -3033,10 +2974,10 @@
         <v>3</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="I1" s="2" t="s">
         <v>20</v>
@@ -3070,7 +3011,7 @@
     <col min="14" max="14" width="20" style="1" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="16.7109375" style="1" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="19" style="1" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="15.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="34.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="27.28515625" style="1" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="24.140625" style="1" bestFit="1" customWidth="1"/>
     <col min="20" max="16384" width="9.140625" style="1"/>
@@ -3078,7 +3019,7 @@
   <sheetData>
     <row r="1" spans="1:19" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>58</v>
@@ -3090,10 +3031,10 @@
         <v>55</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>119</v>
+        <v>109</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>21</v>
@@ -3105,7 +3046,7 @@
         <v>23</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>88</v>
+        <v>82</v>
       </c>
       <c r="K1" s="2" t="s">
         <v>24</v>
@@ -3164,7 +3105,7 @@
   <sheetData>
     <row r="1" spans="1:13" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>89</v>
+        <v>83</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>58</v>
@@ -3176,13 +3117,13 @@
         <v>55</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>119</v>
+        <v>109</v>
       </c>
       <c r="F1" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="G1" s="2" t="s">
         <v>68</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>69</v>
       </c>
       <c r="H1" s="2" t="s">
         <v>4</v>
@@ -3228,7 +3169,7 @@
   <sheetData>
     <row r="1" spans="1:10" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>111</v>
+        <v>101</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>58</v>
@@ -3237,13 +3178,13 @@
         <v>59</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>112</v>
+        <v>102</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>36</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>113</v>
+        <v>103</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>37</v>
@@ -3255,7 +3196,7 @@
         <v>55</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>119</v>
+        <v>109</v>
       </c>
     </row>
   </sheetData>
@@ -3281,7 +3222,7 @@
   <sheetData>
     <row r="1" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>111</v>
+        <v>101</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>58</v>
@@ -3290,13 +3231,13 @@
         <v>59</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>112</v>
+        <v>102</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>36</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>113</v>
+        <v>103</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>37</v>
@@ -3308,7 +3249,7 @@
         <v>55</v>
       </c>
       <c r="J1" s="3" t="s">
-        <v>119</v>
+        <v>109</v>
       </c>
     </row>
   </sheetData>
@@ -3323,7 +3264,7 @@
   <dimension ref="A1:H1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="54" style="1" customWidth="1"/>
+    <col min="1" max="1" width="76.85546875" style="1" customWidth="1"/>
     <col min="2" max="2" width="31.42578125" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="32" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="20.7109375" style="1" bestFit="1" customWidth="1"/>
@@ -3334,7 +3275,7 @@
   <sheetData>
     <row r="1" spans="1:8" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>111</v>
+        <v>101</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>58</v>
@@ -3343,10 +3284,10 @@
         <v>59</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>112</v>
+        <v>102</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>113</v>
+        <v>103</v>
       </c>
       <c r="F1" s="2" t="s">
         <v>37</v>
@@ -3355,7 +3296,7 @@
         <v>55</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>119</v>
+        <v>109</v>
       </c>
     </row>
   </sheetData>
@@ -3385,7 +3326,7 @@
   <sheetData>
     <row r="1" spans="1:12" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>58</v>
@@ -3397,13 +3338,13 @@
         <v>39</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>116</v>
+        <v>106</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>114</v>
+        <v>104</v>
       </c>
       <c r="H1" s="2" t="s">
         <v>40</v>
@@ -3418,7 +3359,7 @@
         <v>55</v>
       </c>
       <c r="L1" s="2" t="s">
-        <v>119</v>
+        <v>109</v>
       </c>
     </row>
   </sheetData>
@@ -3447,7 +3388,7 @@
   <sheetData>
     <row r="1" spans="1:10" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>58</v>
@@ -3456,7 +3397,7 @@
         <v>59</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>11</v>
@@ -3465,16 +3406,16 @@
         <v>55</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>119</v>
+        <v>109</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(Feat-B-005): Import Employees new mandatory field and field changes #3
</commit_message>
<xml_diff>
--- a/public/template_excel/DATA PEGAWAI ASN.xlsx
+++ b/public/template_excel/DATA PEGAWAI ASN.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7755" firstSheet="12" activeTab="16"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7755"/>
   </bookViews>
   <sheets>
     <sheet name="Data Pegawai" sheetId="1" r:id="rId1"/>
@@ -1947,9 +1947,6 @@
     <t>Keterangan Lainnya</t>
   </si>
   <si>
-    <t>Jenis Pegawai</t>
-  </si>
-  <si>
     <t>Instansi Induk</t>
   </si>
   <si>
@@ -1974,9 +1971,6 @@
     <t>Masa Kerja Golongan Jumlah Bulan</t>
   </si>
   <si>
-    <t>Status Pegawai</t>
-  </si>
-  <si>
     <t>No KK</t>
   </si>
   <si>
@@ -1989,7 +1983,13 @@
     <t>Email Dinas *</t>
   </si>
   <si>
-    <t>Kontak Darurat (Nama, Nomor Handphone, Hubungan dengan pegawai)</t>
+    <t>Jenis Pegawai *</t>
+  </si>
+  <si>
+    <t>Status Pegawai *</t>
+  </si>
+  <si>
+    <t>Kontak Darurat (Nama, Nomor Handphone, Hubungan dengan pegawai) *</t>
   </si>
 </sst>
 </file>
@@ -2437,7 +2437,7 @@
         <v>114</v>
       </c>
       <c r="N1" s="2" t="s">
-        <v>115</v>
+        <v>127</v>
       </c>
       <c r="O1" s="2" t="s">
         <v>93</v>
@@ -2464,16 +2464,16 @@
         <v>10</v>
       </c>
       <c r="W1" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="X1" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="X1" s="2" t="s">
+      <c r="Y1" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="Y1" s="2" t="s">
+      <c r="Z1" s="2" t="s">
         <v>118</v>
-      </c>
-      <c r="Z1" s="2" t="s">
-        <v>119</v>
       </c>
       <c r="AA1" s="2" t="s">
         <v>12</v>
@@ -2482,37 +2482,37 @@
         <v>54</v>
       </c>
       <c r="AC1" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="AD1" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="AD1" s="2" t="s">
+      <c r="AE1" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="AE1" s="2" t="s">
+      <c r="AF1" s="2" t="s">
         <v>122</v>
-      </c>
-      <c r="AF1" s="2" t="s">
-        <v>123</v>
       </c>
       <c r="AG1" s="2" t="s">
         <v>13</v>
       </c>
       <c r="AH1" s="2" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="AI1" s="2" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="AJ1" s="2" t="s">
         <v>70</v>
       </c>
       <c r="AK1" s="2" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="AL1" s="2" t="s">
         <v>14</v>
       </c>
       <c r="AM1" s="2" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="AN1" s="2" t="s">
         <v>15</v>
@@ -2530,7 +2530,7 @@
         <v>19</v>
       </c>
       <c r="AS1" s="2" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="AT1" s="2" t="s">
         <v>129</v>

</xml_diff>

<commit_message>
feat(Feat-B-013): adjust Import and Export new columns
</commit_message>
<xml_diff>
--- a/public/template_excel/DATA PEGAWAI ASN.xlsx
+++ b/public/template_excel/DATA PEGAWAI ASN.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7755"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7755" firstSheet="8" activeTab="10"/>
   </bookViews>
   <sheets>
     <sheet name="Data Pegawai" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,7 @@
     <sheet name="Riwayat Golongan" sheetId="3" r:id="rId4"/>
     <sheet name="Riwayat Pelatihan Struktural" sheetId="6" r:id="rId5"/>
     <sheet name="Riwayat Pelatihan Fungsional" sheetId="7" r:id="rId6"/>
-    <sheet name="Riwayat Pelatihan Teknis" sheetId="8" r:id="rId7"/>
+    <sheet name="Riwayat Pelatihan Teknis" sheetId="19" r:id="rId7"/>
     <sheet name="Riwayat Penghargaan" sheetId="9" r:id="rId8"/>
     <sheet name="Riwayat SKP" sheetId="10" r:id="rId9"/>
     <sheet name="Penilaian Prestasi Kerja" sheetId="11" r:id="rId10"/>
@@ -928,7 +928,32 @@
         </r>
       </text>
     </comment>
-    <comment ref="G1" authorId="0" shapeId="0">
+    <comment ref="E1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Wilayah</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+- Dalam Negeri
+- Luar Negeri</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="I1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -1268,6 +1293,35 @@
         </r>
       </text>
     </comment>
+    <comment ref="E1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Jenjang</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+- Pelatihan Kepemimpinan Nasional Tingkat I
+- Pelatihan Kepemimpinan Nasional Tingkat II
+- Pelatihan Kepemimpinan Administrator
+- Pelatihan Kepemimpinan Pengawas
+- Pelatihan Dasar CPNS
+- Pelatihan Lainnya </t>
+        </r>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
@@ -1313,6 +1367,36 @@
         </r>
       </text>
     </comment>
+    <comment ref="E1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Jenjang</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+- Terampil
+- Mahir
+- Penyelia
+- Ahli Pertama
+- Ahli Muda
+- Ahli Madya
+- Ahli Utama</t>
+        </r>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
@@ -1355,6 +1439,61 @@
 - Oktober
 - November
 - Desember</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="I1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Rumpun</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+Pengelolaan Sumber Daya Manusia 
+Kelembagaan dan Tata Laksana
+Pengembangan Kompetensi 
+Bantuan Hukum
+Perencanaan Program dan Anggaran
+Akuntabilitas Kinerja
+Keuangan
+Audit Internal
+Tata Usaha
+Arsip
+Perpustakaan
+Perancangan Grafis
+Pengelolaan Bangunan
+Pengelolaan Kendaraan serta Perlengkapan dan Peralatan
+Kerumahtanggaan/Tata Gerha
+Pengamanan Dalam
+Pelayanan Medis
+Sistem Informasi
+Infrastruktur
+Pengelolaan Informasi Publik
+Peliputan dan Dokumentasi
+Protokol VVIP dan VIP
+Ajudan VVIP dan VIP
+Pengelolaan Benda Seni dan Budaya
+Pengamanan VIP dan VVIP
+Analisis Kebijakan
+Analisis Pengaduan Masyarakat
+Analisis Hukum dan Perundang-undangan
+Kerja Sama Teknik dan Tenaga Asing
+Penetapan Pengangkatan/Pemberhentian/ Pensiun/Cuti bagi Pejabat Negara/Pejabat Pemerintah/Perwira TNI/POLRI
+Penetapan Gelar, Tanda Jasa, dan Tanda Kehormatan
+Perjalanan Dinas Luar Negeri</t>
         </r>
       </text>
     </comment>
@@ -1600,7 +1739,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="203" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="133">
   <si>
     <t>Golongan</t>
   </si>
@@ -1713,9 +1852,6 @@
     <t>Jenjang</t>
   </si>
   <si>
-    <t>Durasi Pelatihan (Hari)</t>
-  </si>
-  <si>
     <t>Penyelenggara</t>
   </si>
   <si>
@@ -1746,9 +1882,6 @@
     <t>Nama Pejabat Berwenang</t>
   </si>
   <si>
-    <t>Uraian</t>
-  </si>
-  <si>
     <t>Nama Bapak</t>
   </si>
   <si>
@@ -1990,6 +2123,21 @@
   </si>
   <si>
     <t>Kontak Darurat (Nama, Nomor Handphone, Hubungan dengan pegawai) *</t>
+  </si>
+  <si>
+    <t>Jam Pelajaran</t>
+  </si>
+  <si>
+    <t>Tanggal Pelaksaanan Selesai</t>
+  </si>
+  <si>
+    <t>Tanggal Pelaksanaan Selesai</t>
+  </si>
+  <si>
+    <t>Wilayah</t>
+  </si>
+  <si>
+    <t>Akreditasi</t>
   </si>
 </sst>
 </file>
@@ -2398,7 +2546,7 @@
   <sheetData>
     <row r="1" spans="1:46" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>7</v>
@@ -2407,112 +2555,112 @@
         <v>8</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>1</v>
       </c>
       <c r="F1" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="H1" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="H1" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="I1" s="2" t="s">
+      <c r="J1" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="N1" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="O1" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="P1" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="Q1" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="R1" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="S1" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="J1" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="K1" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="L1" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="M1" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="N1" s="2" t="s">
-        <v>127</v>
-      </c>
-      <c r="O1" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="P1" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="Q1" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="R1" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="S1" s="2" t="s">
-        <v>67</v>
-      </c>
       <c r="T1" s="2" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="U1" s="2" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="V1" s="2" t="s">
         <v>10</v>
       </c>
       <c r="W1" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="X1" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="Y1" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="X1" s="2" t="s">
+      <c r="Z1" s="2" t="s">
         <v>116</v>
-      </c>
-      <c r="Y1" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="Z1" s="2" t="s">
-        <v>118</v>
       </c>
       <c r="AA1" s="2" t="s">
         <v>12</v>
       </c>
       <c r="AB1" s="2" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="AC1" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="AD1" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="AE1" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="AD1" s="2" t="s">
+      <c r="AF1" s="2" t="s">
         <v>120</v>
-      </c>
-      <c r="AE1" s="2" t="s">
-        <v>121</v>
-      </c>
-      <c r="AF1" s="2" t="s">
-        <v>122</v>
       </c>
       <c r="AG1" s="2" t="s">
         <v>13</v>
       </c>
       <c r="AH1" s="2" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="AI1" s="2" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="AJ1" s="2" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="AK1" s="2" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="AL1" s="2" t="s">
         <v>14</v>
       </c>
       <c r="AM1" s="2" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="AN1" s="2" t="s">
         <v>15</v>
@@ -2530,10 +2678,10 @@
         <v>19</v>
       </c>
       <c r="AS1" s="2" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="AT1" s="2" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
     </row>
     <row r="3" spans="1:46" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -2562,28 +2710,28 @@
   <sheetData>
     <row r="1" spans="1:8" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="G1" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="B1" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>86</v>
-      </c>
       <c r="H1" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
   </sheetData>
@@ -2610,24 +2758,25 @@
     <col min="11" max="11" width="34.28515625" style="1" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="34.7109375" style="1" bestFit="1" customWidth="1"/>
     <col min="13" max="14" width="26.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="15" max="16384" width="9.140625" style="1"/>
+    <col min="15" max="15" width="12.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="16" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="B1" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>59</v>
-      </c>
       <c r="D1" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="F1" s="2" t="s">
         <v>0</v>
@@ -2636,28 +2785,28 @@
         <v>9</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="I1" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="J1" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="K1" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="M1" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="K1" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="L1" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="M1" s="2" t="s">
+      <c r="N1" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="N1" s="2" t="s">
-        <v>47</v>
-      </c>
       <c r="O1" s="2" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
     </row>
   </sheetData>
@@ -2693,58 +2842,58 @@
   <sheetData>
     <row r="1" spans="1:18" s="3" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="C1" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="L1" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="M1" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="E1" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="G1" s="3" t="s">
+      <c r="N1" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="O1" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="P1" s="3" t="s">
         <v>64</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="J1" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="K1" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="L1" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="M1" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="N1" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="O1" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="P1" s="3" t="s">
-        <v>66</v>
       </c>
       <c r="Q1" s="3" t="s">
         <v>16</v>
       </c>
       <c r="R1" s="3" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
     </row>
   </sheetData>
@@ -2772,25 +2921,25 @@
   <sheetData>
     <row r="1" spans="1:7" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="C1" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="E1" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>97</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>99</v>
       </c>
     </row>
   </sheetData>
@@ -2812,13 +2961,13 @@
   <sheetData>
     <row r="1" spans="1:3" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
   </sheetData>
@@ -2842,19 +2991,19 @@
   <sheetData>
     <row r="1" spans="1:5" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
   </sheetData>
@@ -2879,19 +3028,19 @@
   <sheetData>
     <row r="1" spans="1:5" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
   </sheetData>
@@ -2916,19 +3065,19 @@
   <sheetData>
     <row r="1" spans="1:5" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
   </sheetData>
@@ -2939,47 +3088,54 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:K1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.42578125" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="22.42578125" style="1" customWidth="1"/>
     <col min="3" max="3" width="22.5703125" style="1" customWidth="1"/>
     <col min="4" max="4" width="19.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9" style="1" customWidth="1"/>
-    <col min="7" max="7" width="8.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="20.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="16384" width="9.140625" style="1"/>
+    <col min="5" max="6" width="19.28515625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="9" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9" style="1" customWidth="1"/>
+    <col min="9" max="9" width="8.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="20.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="C1" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="J1" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="E1" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="I1" s="2" t="s">
+      <c r="K1" s="2" t="s">
         <v>20</v>
       </c>
     </row>
@@ -3019,22 +3175,22 @@
   <sheetData>
     <row r="1" spans="1:19" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>21</v>
@@ -3046,7 +3202,7 @@
         <v>23</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="K1" s="2" t="s">
         <v>24</v>
@@ -3105,25 +3261,25 @@
   <sheetData>
     <row r="1" spans="1:13" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="H1" s="2" t="s">
         <v>4</v>
@@ -3153,50 +3309,59 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:L1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="31.42578125" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="32" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="20.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.5703125" style="1" customWidth="1"/>
-    <col min="6" max="7" width="23.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="16384" width="9.140625" style="1"/>
+    <col min="5" max="5" width="22.140625" style="1" customWidth="1"/>
+    <col min="6" max="6" width="23.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="29" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="23.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.5703125" style="1" customWidth="1"/>
+    <col min="11" max="11" width="17.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>36</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="G1" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="I1" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="H1" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="I1" s="2" t="s">
-        <v>55</v>
-      </c>
       <c r="J1" s="2" t="s">
-        <v>109</v>
+        <v>42</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>107</v>
       </c>
     </row>
   </sheetData>
@@ -3207,49 +3372,54 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:K1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="53.7109375" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="31.42578125" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="32" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="21.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="7" width="23.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="16384" width="9.140625" style="1"/>
+    <col min="5" max="6" width="23.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="29" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="23.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>36</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="G1" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="I1" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="H1" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="I1" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="J1" s="3" t="s">
-        <v>109</v>
+      <c r="J1" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>107</v>
       </c>
     </row>
   </sheetData>
@@ -3261,42 +3431,53 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:K1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="76.85546875" style="1" customWidth="1"/>
-    <col min="2" max="2" width="31.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="32" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="23.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="17.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="16384" width="9.140625" style="1"/>
+    <col min="1" max="1" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="31.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="32" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="23.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="29" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="E1" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="B1" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>102</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>103</v>
-      </c>
       <c r="F1" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="H1" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="G1" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>109</v>
+      <c r="I1" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>107</v>
       </c>
     </row>
   </sheetData>
@@ -3326,40 +3507,40 @@
   <sheetData>
     <row r="1" spans="1:12" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="D1" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="H1" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="E1" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="H1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="J1" s="2" t="s">
-        <v>42</v>
-      </c>
       <c r="K1" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="L1" s="2" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
   </sheetData>
@@ -3388,34 +3569,34 @@
   <sheetData>
     <row r="1" spans="1:10" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>11</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="H1" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="J1" s="2" t="s">
         <v>89</v>
-      </c>
-      <c r="I1" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="J1" s="2" t="s">
-        <v>91</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix(Fix-B-013): Fixing hapus tanggal terima di Riwayat Penghargaan dan Detail Pegawai #3
</commit_message>
<xml_diff>
--- a/public/template_excel/DATA PEGAWAI ASN.xlsx
+++ b/public/template_excel/DATA PEGAWAI ASN.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7755" firstSheet="8" activeTab="10"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7755" firstSheet="6" activeTab="7"/>
   </bookViews>
   <sheets>
     <sheet name="Data Pegawai" sheetId="1" r:id="rId1"/>
@@ -1507,6 +1507,35 @@
     <author>Windows User</author>
   </authors>
   <commentList>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">Nama Penghargaan
+- </t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Satyalancana Karya Satya 10th
+- Satyalancana Karya Satya 20th
+- Satyalancana Karya Satya 30th
+- Satyalancana Wira Karya
+- Bintang Jasa Utama
+- Penghargaan Lainnya</t>
+        </r>
+      </text>
+    </comment>
     <comment ref="B1" authorId="0" shapeId="0">
       <text>
         <r>
@@ -1739,7 +1768,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="132">
   <si>
     <t>Golongan</t>
   </si>
@@ -1862,9 +1891,6 @@
   </si>
   <si>
     <t>Instansi Pemberi Penghargaan</t>
-  </si>
-  <si>
-    <t>Tanggal Terima</t>
   </si>
   <si>
     <t>Keterangan</t>
@@ -2546,7 +2572,7 @@
   <sheetData>
     <row r="1" spans="1:46" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>7</v>
@@ -2555,112 +2581,112 @@
         <v>8</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>1</v>
       </c>
       <c r="F1" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="G1" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="I1" s="2" t="s">
-        <v>63</v>
-      </c>
       <c r="J1" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="K1" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="L1" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="M1" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="M1" s="2" t="s">
-        <v>112</v>
-      </c>
       <c r="N1" s="2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="O1" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="P1" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="Q1" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="R1" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="S1" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="T1" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="U1" s="2" t="s">
         <v>91</v>
-      </c>
-      <c r="P1" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="Q1" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="R1" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="S1" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="T1" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="U1" s="2" t="s">
-        <v>92</v>
       </c>
       <c r="V1" s="2" t="s">
         <v>10</v>
       </c>
       <c r="W1" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="X1" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="X1" s="2" t="s">
+      <c r="Y1" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="Y1" s="2" t="s">
+      <c r="Z1" s="2" t="s">
         <v>115</v>
-      </c>
-      <c r="Z1" s="2" t="s">
-        <v>116</v>
       </c>
       <c r="AA1" s="2" t="s">
         <v>12</v>
       </c>
       <c r="AB1" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AC1" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="AD1" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="AD1" s="2" t="s">
+      <c r="AE1" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="AE1" s="2" t="s">
+      <c r="AF1" s="2" t="s">
         <v>119</v>
-      </c>
-      <c r="AF1" s="2" t="s">
-        <v>120</v>
       </c>
       <c r="AG1" s="2" t="s">
         <v>13</v>
       </c>
       <c r="AH1" s="2" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="AI1" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="AJ1" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="AK1" s="2" t="s">
         <v>121</v>
-      </c>
-      <c r="AJ1" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="AK1" s="2" t="s">
-        <v>122</v>
       </c>
       <c r="AL1" s="2" t="s">
         <v>14</v>
       </c>
       <c r="AM1" s="2" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="AN1" s="2" t="s">
         <v>15</v>
@@ -2678,10 +2704,10 @@
         <v>19</v>
       </c>
       <c r="AS1" s="2" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="AT1" s="2" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="3" spans="1:46" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -2710,28 +2736,28 @@
   <sheetData>
     <row r="1" spans="1:8" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="B1" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="G1" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="E1" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>84</v>
-      </c>
       <c r="H1" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
   </sheetData>
@@ -2764,19 +2790,19 @@
   <sheetData>
     <row r="1" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="C1" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="C1" s="2" t="s">
-        <v>57</v>
-      </c>
       <c r="D1" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F1" s="2" t="s">
         <v>0</v>
@@ -2785,28 +2811,28 @@
         <v>9</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="I1" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="J1" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="K1" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="M1" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="K1" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="L1" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="M1" s="2" t="s">
+      <c r="N1" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="N1" s="2" t="s">
-        <v>46</v>
-      </c>
       <c r="O1" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
   </sheetData>
@@ -2842,58 +2868,58 @@
   <sheetData>
     <row r="1" spans="1:18" s="3" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C1" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="D1" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="E1" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="L1" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="E1" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="F1" s="3" t="s">
+      <c r="M1" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="N1" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="O1" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="P1" s="3" t="s">
         <v>63</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="J1" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="K1" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="L1" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="M1" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="N1" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="O1" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="P1" s="3" t="s">
-        <v>64</v>
       </c>
       <c r="Q1" s="3" t="s">
         <v>16</v>
       </c>
       <c r="R1" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -2921,25 +2947,25 @@
   <sheetData>
     <row r="1" spans="1:7" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C1" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>96</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>97</v>
       </c>
     </row>
   </sheetData>
@@ -2961,13 +2987,13 @@
   <sheetData>
     <row r="1" spans="1:3" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
   </sheetData>
@@ -2991,16 +3017,16 @@
   <sheetData>
     <row r="1" spans="1:5" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>37</v>
@@ -3028,16 +3054,16 @@
   <sheetData>
     <row r="1" spans="1:5" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>37</v>
@@ -3065,16 +3091,16 @@
   <sheetData>
     <row r="1" spans="1:5" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>37</v>
@@ -3106,22 +3132,22 @@
   <sheetData>
     <row r="1" spans="1:11" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E1" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="F1" s="2" t="s">
         <v>131</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>132</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>2</v>
@@ -3130,10 +3156,10 @@
         <v>3</v>
       </c>
       <c r="I1" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="J1" s="2" t="s">
         <v>70</v>
-      </c>
-      <c r="J1" s="2" t="s">
-        <v>71</v>
       </c>
       <c r="K1" s="2" t="s">
         <v>20</v>
@@ -3175,22 +3201,22 @@
   <sheetData>
     <row r="1" spans="1:19" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="F1" s="2" t="s">
         <v>78</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>79</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>21</v>
@@ -3202,7 +3228,7 @@
         <v>23</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="K1" s="2" t="s">
         <v>24</v>
@@ -3261,25 +3287,25 @@
   <sheetData>
     <row r="1" spans="1:13" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="C1" s="2" t="s">
-        <v>57</v>
-      </c>
       <c r="D1" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F1" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="G1" s="2" t="s">
         <v>65</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>66</v>
       </c>
       <c r="H1" s="2" t="s">
         <v>4</v>
@@ -3328,40 +3354,40 @@
   <sheetData>
     <row r="1" spans="1:12" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>99</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>100</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>36</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="I1" s="2" t="s">
         <v>37</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="L1" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
   </sheetData>
@@ -3389,37 +3415,37 @@
   <sheetData>
     <row r="1" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>99</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>100</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>36</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="I1" s="2" t="s">
         <v>37</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="K1" s="3" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
   </sheetData>
@@ -3447,25 +3473,25 @@
   <sheetData>
     <row r="1" spans="1:11" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="B1" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="E1" s="2" t="s">
-        <v>101</v>
-      </c>
       <c r="F1" s="2" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="H1" s="2" t="s">
         <v>37</v>
@@ -3474,10 +3500,10 @@
         <v>21</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
   </sheetData>
@@ -3488,7 +3514,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L1"/>
+  <dimension ref="A1:K1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.42578125" style="1" bestFit="1" customWidth="1"/>
@@ -3500,32 +3526,31 @@
     <col min="7" max="7" width="22.42578125" style="1" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="16" style="1" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="31.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="16" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="17.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="16384" width="9.140625" style="1"/>
+    <col min="10" max="10" width="17.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>56</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>57</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>38</v>
       </c>
       <c r="E1" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="F1" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="F1" s="2" t="s">
-        <v>104</v>
-      </c>
       <c r="G1" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="H1" s="2" t="s">
         <v>39</v>
@@ -3534,18 +3559,16 @@
         <v>40</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>41</v>
+        <v>52</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="L1" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <legacyDrawing r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -3569,34 +3592,34 @@
   <sheetData>
     <row r="1" spans="1:10" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>85</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>86</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>11</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="H1" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="I1" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>88</v>
-      </c>
-      <c r="J1" s="2" t="s">
-        <v>89</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(Feat-B-037): add marriage_other_notes to families
</commit_message>
<xml_diff>
--- a/public/template_excel/DATA PEGAWAI ASN.xlsx
+++ b/public/template_excel/DATA PEGAWAI ASN.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7755" firstSheet="6" activeTab="7"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7755"/>
   </bookViews>
   <sheets>
     <sheet name="Data Pegawai" sheetId="1" r:id="rId1"/>
@@ -127,7 +127,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="N1" authorId="0" shapeId="0">
+    <comment ref="M1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -154,7 +154,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="Q1" authorId="0" shapeId="0">
+    <comment ref="P1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -184,7 +184,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="S1" authorId="0" shapeId="0">
+    <comment ref="R1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -242,7 +242,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="U1" authorId="0" shapeId="0">
+    <comment ref="T1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -279,7 +279,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="W1" authorId="0" shapeId="0">
+    <comment ref="V1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -329,7 +329,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="X1" authorId="0" shapeId="0">
+    <comment ref="W1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -360,7 +360,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AH1" authorId="0" shapeId="0">
+    <comment ref="AG1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -392,7 +392,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AK1" authorId="0" shapeId="0">
+    <comment ref="AJ1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -2520,7 +2520,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AT3"/>
+  <dimension ref="A1:AS3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.42578125" style="1" bestFit="1" customWidth="1"/>
@@ -2535,42 +2535,41 @@
     <col min="10" max="10" width="21.42578125" style="1" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="20.7109375" style="1" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="24.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="20.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="19.28515625" style="1" customWidth="1"/>
-    <col min="15" max="15" width="21.5703125" style="1" customWidth="1"/>
-    <col min="16" max="16" width="17.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="84.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="17.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="33.140625" style="1" customWidth="1"/>
-    <col min="20" max="20" width="30.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="21" max="22" width="29" style="1" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="28.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="27.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="27.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="31.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="31.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="29" style="1" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="39.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="58.28515625" style="1" customWidth="1"/>
-    <col min="31" max="31" width="36.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="36.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="17.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="23" style="1" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="19.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="36" max="37" width="25.28515625" style="1" customWidth="1"/>
-    <col min="38" max="38" width="73.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="27.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="20" style="1" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="13.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="15.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="19.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="44" max="44" width="16.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="45" max="45" width="15.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="46" max="46" width="73.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="47" max="16384" width="9.140625" style="1"/>
+    <col min="13" max="13" width="19.28515625" style="1" customWidth="1"/>
+    <col min="14" max="14" width="21.5703125" style="1" customWidth="1"/>
+    <col min="15" max="15" width="17.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="84.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="17.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="33.140625" style="1" customWidth="1"/>
+    <col min="19" max="19" width="30.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="20" max="21" width="29" style="1" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="28.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="27.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="27.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="31.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="31.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="29" style="1" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="39.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="58.28515625" style="1" customWidth="1"/>
+    <col min="30" max="30" width="36.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="36.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="17.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="23" style="1" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="19.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="35" max="36" width="25.28515625" style="1" customWidth="1"/>
+    <col min="37" max="37" width="73.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="27.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="20" style="1" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="13.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="15.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="19.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="16.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="44" max="44" width="15.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="73.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="46" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:46" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:45" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>57</v>
       </c>
@@ -2608,109 +2607,106 @@
         <v>110</v>
       </c>
       <c r="M1" s="2" t="s">
-        <v>111</v>
+        <v>124</v>
       </c>
       <c r="N1" s="2" t="s">
-        <v>124</v>
+        <v>90</v>
       </c>
       <c r="O1" s="2" t="s">
-        <v>90</v>
+        <v>107</v>
       </c>
       <c r="P1" s="2" t="s">
-        <v>107</v>
+        <v>78</v>
       </c>
       <c r="Q1" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="R1" s="2" t="s">
-        <v>79</v>
+        <v>64</v>
       </c>
       <c r="S1" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="T1" s="2" t="s">
-        <v>65</v>
+        <v>91</v>
       </c>
       <c r="U1" s="2" t="s">
-        <v>91</v>
+        <v>10</v>
       </c>
       <c r="V1" s="2" t="s">
-        <v>10</v>
+        <v>112</v>
       </c>
       <c r="W1" s="2" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="X1" s="2" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="Y1" s="2" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="Z1" s="2" t="s">
-        <v>115</v>
+        <v>12</v>
       </c>
       <c r="AA1" s="2" t="s">
-        <v>12</v>
+        <v>51</v>
       </c>
       <c r="AB1" s="2" t="s">
-        <v>51</v>
+        <v>116</v>
       </c>
       <c r="AC1" s="2" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="AD1" s="2" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AE1" s="2" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AF1" s="2" t="s">
-        <v>119</v>
+        <v>13</v>
       </c>
       <c r="AG1" s="2" t="s">
-        <v>13</v>
+        <v>125</v>
       </c>
       <c r="AH1" s="2" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="AI1" s="2" t="s">
-        <v>120</v>
+        <v>67</v>
       </c>
       <c r="AJ1" s="2" t="s">
-        <v>67</v>
+        <v>121</v>
       </c>
       <c r="AK1" s="2" t="s">
-        <v>121</v>
+        <v>14</v>
       </c>
       <c r="AL1" s="2" t="s">
-        <v>14</v>
+        <v>122</v>
       </c>
       <c r="AM1" s="2" t="s">
-        <v>122</v>
+        <v>15</v>
       </c>
       <c r="AN1" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="AO1" s="2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="AP1" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="AQ1" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="AR1" s="2" t="s">
-        <v>19</v>
+        <v>123</v>
       </c>
       <c r="AS1" s="2" t="s">
-        <v>123</v>
-      </c>
-      <c r="AT1" s="2" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="3" spans="1:46" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="3" spans="1:45" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -2843,7 +2839,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:R1"/>
+  <dimension ref="A1:S1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.42578125" style="1" bestFit="1" customWidth="1"/>
@@ -2861,12 +2857,13 @@
     <col min="13" max="13" width="25" style="1" bestFit="1" customWidth="1"/>
     <col min="14" max="15" width="24.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="21.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="13.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="14.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="19" max="16384" width="9.140625" style="1"/>
+    <col min="17" max="17" width="21.42578125" style="1" customWidth="1"/>
+    <col min="18" max="18" width="13.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="14.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="20" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" s="3" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:19" s="3" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>52</v>
       </c>
@@ -2916,9 +2913,12 @@
         <v>63</v>
       </c>
       <c r="Q1" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="R1" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="3" t="s">
+      <c r="S1" s="3" t="s">
         <v>50</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(Feat-b-38) mandatory fields import selain pada field Data Pegawai #2
</commit_message>
<xml_diff>
--- a/public/template_excel/DATA PEGAWAI ASN.xlsx
+++ b/public/template_excel/DATA PEGAWAI ASN.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="153222"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27928"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\WORK\simdatuk-dev\public\template_excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\api\public\template_excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0262B83C-5620-4014-821D-CDB303DAC246}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7755"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="10" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Data Pegawai" sheetId="1" r:id="rId1"/>
@@ -40,12 +41,12 @@
 </file>
 
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>Windows User</author>
   </authors>
   <commentList>
-    <comment ref="H1" authorId="0" shapeId="0">
+    <comment ref="H1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000001000000}">
       <text>
         <r>
           <rPr>
@@ -74,7 +75,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="I1" authorId="0" shapeId="0">
+    <comment ref="I1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000002000000}">
       <text>
         <r>
           <rPr>
@@ -99,7 +100,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J1" authorId="0" shapeId="0">
+    <comment ref="J1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000003000000}">
       <text>
         <r>
           <rPr>
@@ -127,7 +128,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="M1" authorId="0" shapeId="0">
+    <comment ref="M1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000004000000}">
       <text>
         <r>
           <rPr>
@@ -154,7 +155,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="P1" authorId="0" shapeId="0">
+    <comment ref="P1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000005000000}">
       <text>
         <r>
           <rPr>
@@ -184,7 +185,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="R1" authorId="0" shapeId="0">
+    <comment ref="R1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000006000000}">
       <text>
         <r>
           <rPr>
@@ -242,7 +243,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="T1" authorId="0" shapeId="0">
+    <comment ref="T1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000007000000}">
       <text>
         <r>
           <rPr>
@@ -279,7 +280,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="V1" authorId="0" shapeId="0">
+    <comment ref="V1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000008000000}">
       <text>
         <r>
           <rPr>
@@ -329,7 +330,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="W1" authorId="0" shapeId="0">
+    <comment ref="W1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000009000000}">
       <text>
         <r>
           <rPr>
@@ -360,7 +361,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AG1" authorId="0" shapeId="0">
+    <comment ref="AG1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000A000000}">
       <text>
         <r>
           <rPr>
@@ -392,7 +393,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AJ1" authorId="0" shapeId="0">
+    <comment ref="AJ1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000B000000}">
       <text>
         <r>
           <rPr>
@@ -430,12 +431,12 @@
 </file>
 
 <file path=xl/comments10.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>Windows User</author>
   </authors>
   <commentList>
-    <comment ref="B1" authorId="0" shapeId="0">
+    <comment ref="B1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0900-000001000000}">
       <text>
         <r>
           <rPr>
@@ -470,7 +471,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="H1" authorId="0" shapeId="0">
+    <comment ref="H1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0900-000002000000}">
       <text>
         <r>
           <rPr>
@@ -503,12 +504,12 @@
 </file>
 
 <file path=xl/comments11.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>Windows User</author>
   </authors>
   <commentList>
-    <comment ref="B1" authorId="0" shapeId="0">
+    <comment ref="B1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0A00-000001000000}">
       <text>
         <r>
           <rPr>
@@ -543,7 +544,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="H1" authorId="0" shapeId="0">
+    <comment ref="H1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0A00-000002000000}">
       <text>
         <r>
           <rPr>
@@ -582,12 +583,12 @@
 </file>
 
 <file path=xl/comments12.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>Windows User</author>
   </authors>
   <commentList>
-    <comment ref="F1" authorId="0" shapeId="0">
+    <comment ref="F1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0B00-000001000000}">
       <text>
         <r>
           <rPr>
@@ -612,7 +613,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="G1" authorId="0" shapeId="0">
+    <comment ref="G1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0B00-000002000000}">
       <text>
         <r>
           <rPr>
@@ -641,7 +642,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="L1" authorId="0" shapeId="0">
+    <comment ref="L1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0B00-000003000000}">
       <text>
         <r>
           <rPr>
@@ -675,7 +676,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="M1" authorId="0" shapeId="0">
+    <comment ref="M1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0B00-000004000000}">
       <text>
         <r>
           <rPr>
@@ -708,7 +709,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="P1" authorId="0" shapeId="0">
+    <comment ref="P1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0B00-000005000000}">
       <text>
         <r>
           <rPr>
@@ -740,12 +741,12 @@
 </file>
 
 <file path=xl/comments13.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>Windows User</author>
   </authors>
   <commentList>
-    <comment ref="E1" authorId="0" shapeId="0">
+    <comment ref="E1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0C00-000001000000}">
       <text>
         <r>
           <rPr>
@@ -779,12 +780,12 @@
 </file>
 
 <file path=xl/comments14.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>Windows User</author>
   </authors>
   <commentList>
-    <comment ref="D1" authorId="0" shapeId="0">
+    <comment ref="D1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0E00-000001000000}">
       <text>
         <r>
           <rPr>
@@ -815,12 +816,12 @@
 </file>
 
 <file path=xl/comments15.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>Windows User</author>
   </authors>
   <commentList>
-    <comment ref="D1" authorId="0" shapeId="0">
+    <comment ref="D1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0F00-000001000000}">
       <text>
         <r>
           <rPr>
@@ -850,12 +851,12 @@
 </file>
 
 <file path=xl/comments16.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>Windows User</author>
   </authors>
   <commentList>
-    <comment ref="D1" authorId="0" shapeId="0">
+    <comment ref="D1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1000-000001000000}">
       <text>
         <r>
           <rPr>
@@ -892,12 +893,12 @@
 </file>
 
 <file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>Windows User</author>
   </authors>
   <commentList>
-    <comment ref="C1" authorId="0" shapeId="0">
+    <comment ref="C1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000001000000}">
       <text>
         <r>
           <rPr>
@@ -928,7 +929,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E1" authorId="0" shapeId="0">
+    <comment ref="E1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000002000000}">
       <text>
         <r>
           <rPr>
@@ -953,7 +954,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="I1" authorId="0" shapeId="0">
+    <comment ref="I1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000003000000}">
       <text>
         <r>
           <rPr>
@@ -986,12 +987,12 @@
 </file>
 
 <file path=xl/comments3.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>Windows User</author>
   </authors>
   <commentList>
-    <comment ref="B1" authorId="0" shapeId="0">
+    <comment ref="B1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000001000000}">
       <text>
         <r>
           <rPr>
@@ -1026,7 +1027,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="H1" authorId="0" shapeId="0">
+    <comment ref="H1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000002000000}">
       <text>
         <r>
           <rPr>
@@ -1055,7 +1056,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="I1" authorId="0" shapeId="0">
+    <comment ref="I1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000003000000}">
       <text>
         <r>
           <rPr>
@@ -1087,12 +1088,12 @@
 </file>
 
 <file path=xl/comments4.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>Windows User</author>
   </authors>
   <commentList>
-    <comment ref="B1" authorId="0" shapeId="0">
+    <comment ref="B1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0300-000001000000}">
       <text>
         <r>
           <rPr>
@@ -1127,7 +1128,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="F1" authorId="0" shapeId="0">
+    <comment ref="F1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0300-000002000000}">
       <text>
         <r>
           <rPr>
@@ -1184,7 +1185,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="I1" authorId="0" shapeId="0">
+    <comment ref="I1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0300-000003000000}">
       <text>
         <r>
           <rPr>
@@ -1223,7 +1224,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="M1" authorId="0" shapeId="0">
+    <comment ref="M1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0300-000004000000}">
       <text>
         <r>
           <rPr>
@@ -1253,12 +1254,12 @@
 </file>
 
 <file path=xl/comments5.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>Windows User</author>
   </authors>
   <commentList>
-    <comment ref="B1" authorId="0" shapeId="0">
+    <comment ref="B1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0400-000001000000}">
       <text>
         <r>
           <rPr>
@@ -1293,7 +1294,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E1" authorId="0" shapeId="0">
+    <comment ref="E1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0400-000002000000}">
       <text>
         <r>
           <rPr>
@@ -1327,12 +1328,12 @@
 </file>
 
 <file path=xl/comments6.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>Windows User</author>
   </authors>
   <commentList>
-    <comment ref="B1" authorId="0" shapeId="0">
+    <comment ref="B1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0500-000001000000}">
       <text>
         <r>
           <rPr>
@@ -1367,7 +1368,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E1" authorId="0" shapeId="0">
+    <comment ref="E1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0500-000002000000}">
       <text>
         <r>
           <rPr>
@@ -1402,12 +1403,12 @@
 </file>
 
 <file path=xl/comments7.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>Windows User</author>
   </authors>
   <commentList>
-    <comment ref="B1" authorId="0" shapeId="0">
+    <comment ref="B1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0600-000001000000}">
       <text>
         <r>
           <rPr>
@@ -1442,7 +1443,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="I1" authorId="0" shapeId="0">
+    <comment ref="I1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0600-000002000000}">
       <text>
         <r>
           <rPr>
@@ -1502,12 +1503,12 @@
 </file>
 
 <file path=xl/comments8.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>Windows User</author>
   </authors>
   <commentList>
-    <comment ref="A1" authorId="0" shapeId="0">
+    <comment ref="A1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0700-000001000000}">
       <text>
         <r>
           <rPr>
@@ -1536,7 +1537,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B1" authorId="0" shapeId="0">
+    <comment ref="B1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0700-000002000000}">
       <text>
         <r>
           <rPr>
@@ -1571,7 +1572,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E1" authorId="0" shapeId="0">
+    <comment ref="E1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0700-000003000000}">
       <text>
         <r>
           <rPr>
@@ -1615,12 +1616,12 @@
 </file>
 
 <file path=xl/comments9.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>Windows User</author>
   </authors>
   <commentList>
-    <comment ref="B1" authorId="0" shapeId="0">
+    <comment ref="B1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0800-000001000000}">
       <text>
         <r>
           <rPr>
@@ -1655,7 +1656,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D1" authorId="0" shapeId="0">
+    <comment ref="D1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0800-000002000000}">
       <text>
         <r>
           <rPr>
@@ -1683,7 +1684,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="H1" authorId="0" shapeId="0">
+    <comment ref="H1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0800-000003000000}">
       <text>
         <r>
           <rPr>
@@ -1709,7 +1710,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="I1" authorId="0" shapeId="0">
+    <comment ref="I1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0800-000004000000}">
       <text>
         <r>
           <rPr>
@@ -1737,7 +1738,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J1" authorId="0" shapeId="0">
+    <comment ref="J1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0800-000005000000}">
       <text>
         <r>
           <rPr>
@@ -1768,7 +1769,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="139">
   <si>
     <t>Golongan</t>
   </si>
@@ -1929,18 +1930,6 @@
     <t>NIK *</t>
   </si>
   <si>
-    <t>Jenis Hukuman *</t>
-  </si>
-  <si>
-    <t>Nama Riwayat Hukuman Disiplin *</t>
-  </si>
-  <si>
-    <t>Bulan Periode Input Riwayat *</t>
-  </si>
-  <si>
-    <t>Tahun Periode Input Riwayat *</t>
-  </si>
-  <si>
     <t>Nama *</t>
   </si>
   <si>
@@ -1959,135 +1948,27 @@
     <t>Jenis Kelamin *</t>
   </si>
   <si>
-    <t>Status Perkawinan *</t>
-  </si>
-  <si>
     <t>Golongan *</t>
   </si>
   <si>
     <t>TMT Golongan *</t>
   </si>
   <si>
-    <t>Tingkat *</t>
-  </si>
-  <si>
     <t>No NIK *</t>
   </si>
   <si>
-    <t>Nama Sekolah *</t>
-  </si>
-  <si>
-    <t>Status *</t>
-  </si>
-  <si>
-    <t>Tahun Lulus *</t>
-  </si>
-  <si>
-    <t>No Kartu Keluarga *</t>
-  </si>
-  <si>
-    <t>Nama Anggota Keluarga *</t>
-  </si>
-  <si>
-    <t>Hubungan Keluarga *</t>
-  </si>
-  <si>
-    <t>Pendidikan *</t>
-  </si>
-  <si>
-    <t>Catatan *</t>
-  </si>
-  <si>
-    <t>Hasil *</t>
-  </si>
-  <si>
-    <t>Nama Riwayat Jabatan *</t>
-  </si>
-  <si>
     <t>Jabatan *</t>
   </si>
   <si>
     <t>TMT Menjabat *</t>
   </si>
   <si>
-    <t>Nama Riwayat Golongan *</t>
-  </si>
-  <si>
-    <t>Nama Riwayat PPK *</t>
-  </si>
-  <si>
-    <t>Periode PPK *</t>
-  </si>
-  <si>
-    <t>Nilai Prestasi Kerja *</t>
-  </si>
-  <si>
-    <t>Nama Riwayat SKP *</t>
-  </si>
-  <si>
-    <t>Periode Penilaian *</t>
-  </si>
-  <si>
-    <t>Rating Perilaku Kerja *</t>
-  </si>
-  <si>
-    <t>Predikat Kinerja Pegawai *</t>
-  </si>
-  <si>
-    <t>Capaian Kinerja Organisasi *</t>
-  </si>
-  <si>
-    <t>Nama Penghargaan *</t>
-  </si>
-  <si>
     <t>TMT CPNS *</t>
   </si>
   <si>
     <t>Eselon</t>
   </si>
   <si>
-    <t>Tanggal Awal Cuti *</t>
-  </si>
-  <si>
-    <t>Tanggal Akhir Cuti *</t>
-  </si>
-  <si>
-    <t>Jenis Cuti *</t>
-  </si>
-  <si>
-    <t>No Cuti *</t>
-  </si>
-  <si>
-    <t>Keterangan *</t>
-  </si>
-  <si>
-    <t>Tanggal *</t>
-  </si>
-  <si>
-    <t>Nama Diklat *</t>
-  </si>
-  <si>
-    <t>No Surat Perintah *</t>
-  </si>
-  <si>
-    <t>Tanggal Pelaksanaan *</t>
-  </si>
-  <si>
-    <t>No SK Penghargaan *</t>
-  </si>
-  <si>
-    <t>Jenis SK *</t>
-  </si>
-  <si>
-    <t>Tanggal SK *</t>
-  </si>
-  <si>
-    <t>Tanggal Awal Hukuman Disiplin *</t>
-  </si>
-  <si>
-    <t>Tanggal Akhir Hukuman Disiplin *</t>
-  </si>
-  <si>
     <t>Nama</t>
   </si>
   <si>
@@ -2164,12 +2045,153 @@
   </si>
   <si>
     <t>Akreditasi</t>
+  </si>
+  <si>
+    <t>Tingkat</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nama Sekolah </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Status </t>
+  </si>
+  <si>
+    <t xml:space="preserve">TMT Menjabat </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nama Riwayat Jabatan </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bulan Periode Input Riwayat </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tahun Periode Input Riwayat </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nama Riwayat Golongan </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Golongan </t>
+  </si>
+  <si>
+    <t xml:space="preserve">TMT Golongan </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tanggal </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hasil </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Catatan </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tanggal Awal Cuti </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tanggal Akhir Cuti </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jenis Cuti </t>
+  </si>
+  <si>
+    <t xml:space="preserve">No Cuti </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keterangan </t>
+  </si>
+  <si>
+    <t xml:space="preserve">No Kartu Keluarga </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nama Anggota Keluarga </t>
+  </si>
+  <si>
+    <t xml:space="preserve">No NIK </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jenis Kelamin </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Agama </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tempat Lahir </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tanggal Lahir </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hubungan Keluarga </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pendidikan </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Status Perkawinan </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nama Riwayat Hukuman Disiplin </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jenis Hukuman </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tanggal Awal Hukuman Disiplin </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tanggal Akhir Hukuman Disiplin </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nama Riwayat PPK </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Periode PPK </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nilai Prestasi Kerja </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nama Riwayat SKP </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Periode Penilaian </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rating Perilaku Kerja </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Predikat Kinerja Pegawai </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Capaian Kinerja Organisasi </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nama Penghargaan </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jenis SK </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tanggal SK </t>
+  </si>
+  <si>
+    <t xml:space="preserve">No SK Penghargaan </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nama Diklat </t>
+  </si>
+  <si>
+    <t xml:space="preserve">No Surat Perintah </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tanggal Pelaksanaan </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -2519,59 +2541,59 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AS3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="22.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="22.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="22.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.5546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.5546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="22.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.88671875" style="1" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="12" style="1" customWidth="1"/>
-    <col min="9" max="9" width="15.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="21.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="20.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="24.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="19.28515625" style="1" customWidth="1"/>
-    <col min="14" max="14" width="21.5703125" style="1" customWidth="1"/>
-    <col min="15" max="15" width="17.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="84.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="17.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="33.140625" style="1" customWidth="1"/>
-    <col min="19" max="19" width="30.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="21.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="20.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="24.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="19.33203125" style="1" customWidth="1"/>
+    <col min="14" max="14" width="21.5546875" style="1" customWidth="1"/>
+    <col min="15" max="15" width="17.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="84.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="17.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="33.109375" style="1" customWidth="1"/>
+    <col min="19" max="19" width="30.44140625" style="1" bestFit="1" customWidth="1"/>
     <col min="20" max="21" width="29" style="1" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="28.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="27.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="27.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="31.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="31.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="28.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="27.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="27.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="31.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="31.33203125" style="1" bestFit="1" customWidth="1"/>
     <col min="27" max="27" width="29" style="1" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="39.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="58.28515625" style="1" customWidth="1"/>
-    <col min="30" max="30" width="36.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="36.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="17.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="39.5546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="58.33203125" style="1" customWidth="1"/>
+    <col min="30" max="30" width="36.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="36.109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="17.33203125" style="1" bestFit="1" customWidth="1"/>
     <col min="33" max="33" width="23" style="1" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="19.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="35" max="36" width="25.28515625" style="1" customWidth="1"/>
-    <col min="37" max="37" width="73.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="27.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="19.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="35" max="36" width="25.33203125" style="1" customWidth="1"/>
+    <col min="37" max="37" width="73.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="27.88671875" style="1" bestFit="1" customWidth="1"/>
     <col min="39" max="39" width="20" style="1" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="13.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="15.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="19.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="16.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="44" max="44" width="15.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="45" max="45" width="73.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="46" max="16384" width="9.140625" style="1"/>
+    <col min="40" max="40" width="13.109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="15.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="19.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="16.109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="44" max="44" width="15.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="73.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="46" max="16384" width="9.109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:45" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:45" s="2" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>7</v>
@@ -2580,70 +2602,70 @@
         <v>8</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>1</v>
       </c>
       <c r="F1" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="N1" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="O1" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="P1" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="Q1" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="R1" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="S1" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="H1" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="I1" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="J1" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="K1" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="L1" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="M1" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="N1" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="O1" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="P1" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="Q1" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="R1" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="S1" s="2" t="s">
+      <c r="T1" s="2" t="s">
         <v>65</v>
-      </c>
-      <c r="T1" s="2" t="s">
-        <v>91</v>
       </c>
       <c r="U1" s="2" t="s">
         <v>10</v>
       </c>
       <c r="V1" s="2" t="s">
-        <v>112</v>
+        <v>72</v>
       </c>
       <c r="W1" s="2" t="s">
-        <v>113</v>
+        <v>73</v>
       </c>
       <c r="X1" s="2" t="s">
-        <v>114</v>
+        <v>74</v>
       </c>
       <c r="Y1" s="2" t="s">
-        <v>115</v>
+        <v>75</v>
       </c>
       <c r="Z1" s="2" t="s">
         <v>12</v>
@@ -2652,37 +2674,37 @@
         <v>51</v>
       </c>
       <c r="AB1" s="2" t="s">
-        <v>116</v>
+        <v>76</v>
       </c>
       <c r="AC1" s="2" t="s">
-        <v>117</v>
+        <v>77</v>
       </c>
       <c r="AD1" s="2" t="s">
-        <v>118</v>
+        <v>78</v>
       </c>
       <c r="AE1" s="2" t="s">
-        <v>119</v>
+        <v>79</v>
       </c>
       <c r="AF1" s="2" t="s">
         <v>13</v>
       </c>
       <c r="AG1" s="2" t="s">
-        <v>125</v>
+        <v>85</v>
       </c>
       <c r="AH1" s="2" t="s">
-        <v>120</v>
+        <v>80</v>
       </c>
       <c r="AI1" s="2" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="AJ1" s="2" t="s">
-        <v>121</v>
+        <v>81</v>
       </c>
       <c r="AK1" s="2" t="s">
         <v>14</v>
       </c>
       <c r="AL1" s="2" t="s">
-        <v>122</v>
+        <v>82</v>
       </c>
       <c r="AM1" s="2" t="s">
         <v>15</v>
@@ -2700,13 +2722,13 @@
         <v>19</v>
       </c>
       <c r="AR1" s="2" t="s">
-        <v>123</v>
+        <v>83</v>
       </c>
       <c r="AS1" s="2" t="s">
-        <v>126</v>
+        <v>86</v>
       </c>
     </row>
-    <row r="3" spans="1:45" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="3" spans="1:45" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -2715,42 +2737,42 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <dimension ref="A1:H1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="24.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="31.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="24.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="31.44140625" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="32" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="24.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="24.7109375" style="1" customWidth="1"/>
-    <col min="7" max="7" width="21.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="18.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="16384" width="9.140625" style="1"/>
+    <col min="4" max="4" width="18.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="24.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="24.6640625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="21.109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="16384" width="9.109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" s="2" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>81</v>
+        <v>124</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>55</v>
+        <v>97</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>56</v>
+        <v>98</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>82</v>
+        <v>125</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>52</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>106</v>
+        <v>66</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>83</v>
+        <v>126</v>
       </c>
       <c r="H1" s="2" t="s">
         <v>41</v>
@@ -2763,42 +2785,42 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <dimension ref="A1:O1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="35.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="31.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="35.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="31.44140625" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="32" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17.28515625" style="1" customWidth="1"/>
-    <col min="6" max="6" width="22.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="26.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="25.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.33203125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="22.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.5546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="26.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="25.6640625" style="1" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="30" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="34.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="34.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="13" max="14" width="26.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="16" max="16384" width="9.140625" style="1"/>
+    <col min="11" max="11" width="34.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="34.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="13" max="14" width="26.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="16" max="16384" width="9.109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>54</v>
+        <v>120</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>55</v>
+        <v>97</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>56</v>
+        <v>98</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>52</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>106</v>
+        <v>66</v>
       </c>
       <c r="F1" s="2" t="s">
         <v>0</v>
@@ -2807,7 +2829,7 @@
         <v>9</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>53</v>
+        <v>121</v>
       </c>
       <c r="I1" s="2" t="s">
         <v>42</v>
@@ -2816,10 +2838,10 @@
         <v>43</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>104</v>
+        <v>122</v>
       </c>
       <c r="L1" s="2" t="s">
-        <v>105</v>
+        <v>123</v>
       </c>
       <c r="M1" s="2" t="s">
         <v>44</v>
@@ -2838,58 +2860,58 @@
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
   <dimension ref="A1:S1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="22.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.42578125" style="1" customWidth="1"/>
+    <col min="1" max="1" width="22.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.44140625" style="1" customWidth="1"/>
     <col min="3" max="3" width="21" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="27" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="22.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="22.44140625" style="1" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="25" style="1" bestFit="1" customWidth="1"/>
-    <col min="14" max="15" width="24.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="21.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="21.42578125" style="1" customWidth="1"/>
-    <col min="18" max="18" width="13.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="14.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="20" max="16384" width="9.140625" style="1"/>
+    <col min="14" max="15" width="24.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="21.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="21.44140625" style="1" customWidth="1"/>
+    <col min="18" max="18" width="13.109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="14.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="20" max="16384" width="9.109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" s="3" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:19" s="3" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>52</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>106</v>
+        <v>66</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>71</v>
+        <v>110</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>72</v>
+        <v>111</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>67</v>
+        <v>112</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>62</v>
+        <v>113</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>61</v>
+        <v>114</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>59</v>
+        <v>115</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>60</v>
+        <v>116</v>
       </c>
       <c r="J1" s="3" t="s">
         <v>46</v>
@@ -2898,10 +2920,10 @@
         <v>47</v>
       </c>
       <c r="L1" s="3" t="s">
-        <v>73</v>
+        <v>117</v>
       </c>
       <c r="M1" s="3" t="s">
-        <v>74</v>
+        <v>118</v>
       </c>
       <c r="N1" s="3" t="s">
         <v>48</v>
@@ -2910,10 +2932,10 @@
         <v>49</v>
       </c>
       <c r="P1" s="3" t="s">
-        <v>63</v>
+        <v>119</v>
       </c>
       <c r="Q1" s="3" t="s">
-        <v>111</v>
+        <v>71</v>
       </c>
       <c r="R1" s="3" t="s">
         <v>16</v>
@@ -2930,42 +2952,42 @@
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
   <dimension ref="A1:G1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="22.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.42578125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="21.140625" style="1" customWidth="1"/>
-    <col min="4" max="4" width="21.7109375" style="1" customWidth="1"/>
-    <col min="5" max="5" width="29.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.140625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="16.28515625" style="1" customWidth="1"/>
-    <col min="8" max="8" width="10.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="16384" width="9.140625" style="1"/>
+    <col min="1" max="1" width="22.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.44140625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="21.109375" style="1" customWidth="1"/>
+    <col min="4" max="4" width="21.6640625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="29.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.109375" style="1" customWidth="1"/>
+    <col min="7" max="7" width="16.33203125" style="1" customWidth="1"/>
+    <col min="8" max="8" width="10.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="16384" width="9.109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" s="2" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>52</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="C1" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>93</v>
-      </c>
       <c r="E1" s="2" t="s">
-        <v>94</v>
+        <v>107</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>95</v>
+        <v>108</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>96</v>
+        <v>109</v>
       </c>
     </row>
   </sheetData>
@@ -2975,25 +2997,25 @@
 </file>
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0D00-000000000000}">
   <dimension ref="A1:C1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="22.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.42578125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="23.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="16384" width="9.140625" style="1"/>
+    <col min="1" max="1" width="22.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.44140625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="23.5546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="16384" width="9.109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" s="2" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>52</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>106</v>
+        <v>66</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>75</v>
+        <v>104</v>
       </c>
     </row>
   </sheetData>
@@ -3002,31 +3024,31 @@
 </file>
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0E00-000000000000}">
   <dimension ref="A1:E1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="22.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.42578125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="10.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="22.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="22.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.44140625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="10.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22.6640625" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="18" style="1" customWidth="1"/>
-    <col min="6" max="6" width="16.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="16384" width="9.140625" style="1"/>
+    <col min="6" max="6" width="16.109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="16384" width="9.109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" s="2" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>52</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>106</v>
+        <v>66</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>76</v>
+        <v>103</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>37</v>
@@ -3039,31 +3061,31 @@
 </file>
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0F00-000000000000}">
   <dimension ref="A1:E1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="22.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.42578125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="10.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.28515625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="15.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="16384" width="9.140625" style="1"/>
+    <col min="1" max="1" width="22.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.44140625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="10.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.33203125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="15.5546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="16384" width="9.109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" s="2" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>52</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>106</v>
+        <v>66</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>76</v>
+        <v>103</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>37</v>
@@ -3076,31 +3098,31 @@
 </file>
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1000-000000000000}">
   <dimension ref="A1:E1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="22.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.42578125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="10.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="22.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18.28515625" style="1" customWidth="1"/>
-    <col min="6" max="6" width="16.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="16384" width="9.140625" style="1"/>
+    <col min="1" max="1" width="22.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.44140625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="10.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.33203125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="16.109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="16384" width="9.109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" s="2" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>52</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>106</v>
+        <v>66</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>76</v>
+        <v>103</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>37</v>
@@ -3113,41 +3135,41 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:K1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="22.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.42578125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="22.5703125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="19.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="19.28515625" style="1" customWidth="1"/>
+    <col min="1" max="1" width="22.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.44140625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="22.5546875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="19.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="19.33203125" style="1" customWidth="1"/>
     <col min="7" max="7" width="9" style="1" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="9" style="1" customWidth="1"/>
-    <col min="9" max="9" width="8.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="14.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="20.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="16384" width="9.140625" style="1"/>
+    <col min="9" max="9" width="8.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.5546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="20.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="16384" width="9.109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" s="2" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>52</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>106</v>
+        <v>66</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>66</v>
+        <v>92</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>68</v>
+        <v>93</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>130</v>
+        <v>90</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>131</v>
+        <v>91</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>2</v>
@@ -3156,10 +3178,10 @@
         <v>3</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>69</v>
+        <v>94</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="K1" s="2" t="s">
         <v>20</v>
@@ -3173,50 +3195,50 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:S1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="31.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="31.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="31.5546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="31.44140625" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="32" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="22.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="22.42578125" style="1" customWidth="1"/>
-    <col min="6" max="6" width="31.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="24.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="16.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="20.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="22.44140625" style="1" customWidth="1"/>
+    <col min="6" max="6" width="31.5546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="24.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.5546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="20.6640625" style="1" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="20" style="1" customWidth="1"/>
-    <col min="11" max="11" width="11.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="16.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="15.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.5546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="16.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="15.109375" style="1" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="20" style="1" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="16.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="16.6640625" style="1" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="19" style="1" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="34.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="27.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="24.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="20" max="16384" width="9.140625" style="1"/>
+    <col min="17" max="17" width="34.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="27.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="24.109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="20" max="16384" width="9.109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:19" s="2" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>77</v>
+        <v>96</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>55</v>
+        <v>97</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>56</v>
+        <v>98</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>52</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>106</v>
+        <v>66</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>78</v>
+        <v>9</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>21</v>
@@ -3228,7 +3250,7 @@
         <v>23</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>79</v>
+        <v>95</v>
       </c>
       <c r="K1" s="2" t="s">
         <v>24</v>
@@ -3265,47 +3287,47 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:M1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="32.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="31.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="32.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="31.44140625" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="32" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17.28515625" style="1" customWidth="1"/>
-    <col min="6" max="6" width="18.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="17.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.33203125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="18.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.6640625" style="1" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="22" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="22.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="22.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.44140625" style="1" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="22" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="22.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="17.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="14" max="16384" width="9.140625" style="1"/>
+    <col min="12" max="12" width="22.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="17.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="14" max="16384" width="9.109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" s="2" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>80</v>
+        <v>99</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>55</v>
+        <v>97</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>56</v>
+        <v>98</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>52</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>106</v>
+        <v>66</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>64</v>
+        <v>100</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>65</v>
+        <v>101</v>
       </c>
       <c r="H1" s="2" t="s">
         <v>4</v>
@@ -3334,48 +3356,48 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:L1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="26" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="31.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="31.44140625" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="32" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="22.140625" style="1" customWidth="1"/>
-    <col min="6" max="6" width="23.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="22.109375" style="1" customWidth="1"/>
+    <col min="6" max="6" width="23.44140625" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="29" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="23.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="15.5703125" style="1" customWidth="1"/>
-    <col min="11" max="11" width="17.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="16384" width="9.140625" style="1"/>
+    <col min="8" max="8" width="23.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.5546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.5546875" style="1" customWidth="1"/>
+    <col min="11" max="11" width="17.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="16384" width="9.109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" s="2" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="B1" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>56</v>
-      </c>
       <c r="D1" s="2" t="s">
-        <v>99</v>
+        <v>137</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>36</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>100</v>
+        <v>138</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>129</v>
+        <v>89</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>127</v>
+        <v>87</v>
       </c>
       <c r="I1" s="2" t="s">
         <v>37</v>
@@ -3387,7 +3409,7 @@
         <v>52</v>
       </c>
       <c r="L1" s="2" t="s">
-        <v>106</v>
+        <v>66</v>
       </c>
     </row>
   </sheetData>
@@ -3397,46 +3419,46 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:K1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="53.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="31.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="53.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="31.44140625" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="32" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="23.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="23.44140625" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="29" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="23.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="16384" width="9.140625" style="1"/>
+    <col min="8" max="8" width="23.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.5546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="16384" width="9.109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="B1" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>56</v>
-      </c>
       <c r="D1" s="2" t="s">
-        <v>99</v>
+        <v>137</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>36</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>100</v>
+        <v>138</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>128</v>
+        <v>88</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>127</v>
+        <v>87</v>
       </c>
       <c r="I1" s="2" t="s">
         <v>37</v>
@@ -3445,7 +3467,7 @@
         <v>52</v>
       </c>
       <c r="K1" s="3" t="s">
-        <v>106</v>
+        <v>66</v>
       </c>
     </row>
   </sheetData>
@@ -3456,42 +3478,42 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:K1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="31.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="31.44140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="32" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="23.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="23.44140625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.5703125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15.5703125" customWidth="1"/>
+    <col min="7" max="7" width="14.5546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.5546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" s="2" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="B1" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>56</v>
-      </c>
       <c r="D1" s="2" t="s">
-        <v>99</v>
+        <v>137</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>100</v>
+        <v>138</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>129</v>
+        <v>89</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>127</v>
+        <v>87</v>
       </c>
       <c r="H1" s="2" t="s">
         <v>37</v>
@@ -3503,7 +3525,7 @@
         <v>52</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>106</v>
+        <v>66</v>
       </c>
     </row>
   </sheetData>
@@ -3513,44 +3535,44 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:K1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="22.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="31.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="22.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="31.44140625" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="32" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="52.140625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="34.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="22.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="52.109375" style="1" customWidth="1"/>
+    <col min="5" max="5" width="34.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="22.44140625" style="1" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="16" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="31.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="16384" width="9.140625" style="1"/>
+    <col min="9" max="9" width="31.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="16384" width="9.109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" s="2" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>89</v>
+        <v>132</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>55</v>
+        <v>97</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>56</v>
+        <v>98</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>38</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>102</v>
+        <v>133</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>103</v>
+        <v>134</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>101</v>
+        <v>135</v>
       </c>
       <c r="H1" s="2" t="s">
         <v>39</v>
@@ -3562,7 +3584,7 @@
         <v>52</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>106</v>
+        <v>66</v>
       </c>
     </row>
   </sheetData>
@@ -3573,35 +3595,35 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1:J1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="27.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="31.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="27.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="31.44140625" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="32" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="26" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.85546875" style="1" customWidth="1"/>
-    <col min="6" max="6" width="17.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="17.28515625" style="1" customWidth="1"/>
-    <col min="8" max="8" width="23.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="27.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.88671875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="17.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.33203125" style="1" customWidth="1"/>
+    <col min="8" max="8" width="23.5546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="27.6640625" style="1" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="29" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="16384" width="9.140625" style="1"/>
+    <col min="11" max="16384" width="9.109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" s="2" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>84</v>
+        <v>127</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>55</v>
+        <v>97</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>56</v>
+        <v>98</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>85</v>
+        <v>128</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>11</v>
@@ -3610,16 +3632,16 @@
         <v>52</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>106</v>
+        <v>66</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>86</v>
+        <v>129</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>87</v>
+        <v>130</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>88</v>
+        <v>131</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
[Feat-b-039] hapus kolom status lulus di Riwayat Pendidikan Data Pegawai
</commit_message>
<xml_diff>
--- a/public/template_excel/DATA PEGAWAI ASN.xlsx
+++ b/public/template_excel/DATA PEGAWAI ASN.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\api\public\template_excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0262B83C-5620-4014-821D-CDB303DAC246}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E86E771C-D997-49DF-B8F7-4D80652BB313}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="10" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Data Pegawai" sheetId="1" r:id="rId1"/>
@@ -954,34 +954,6 @@
         </r>
       </text>
     </comment>
-    <comment ref="I1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000003000000}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Status</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-- Lulus
-- DO
-- Aktif
-- Non-aktif
-- Mengundurkan Diri</t>
-        </r>
-      </text>
-    </comment>
   </commentList>
 </comments>
 </file>
@@ -1769,7 +1741,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="139">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="138">
   <si>
     <t>Golongan</t>
   </si>
@@ -2051,9 +2023,6 @@
   </si>
   <si>
     <t xml:space="preserve">Nama Sekolah </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Status </t>
   </si>
   <si>
     <t xml:space="preserve">TMT Menjabat </t>
@@ -2754,16 +2723,16 @@
   <sheetData>
     <row r="1" spans="1:8" s="2" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>124</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>125</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>52</v>
@@ -2772,7 +2741,7 @@
         <v>66</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="H1" s="2" t="s">
         <v>41</v>
@@ -2808,13 +2777,13 @@
   <sheetData>
     <row r="1" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>97</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>98</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>52</v>
@@ -2829,7 +2798,7 @@
         <v>9</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="I1" s="2" t="s">
         <v>42</v>
@@ -2838,10 +2807,10 @@
         <v>43</v>
       </c>
       <c r="K1" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="L1" s="2" t="s">
         <v>122</v>
-      </c>
-      <c r="L1" s="2" t="s">
-        <v>123</v>
       </c>
       <c r="M1" s="2" t="s">
         <v>44</v>
@@ -2893,25 +2862,25 @@
         <v>66</v>
       </c>
       <c r="C1" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="D1" s="3" t="s">
         <v>110</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="E1" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="F1" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="G1" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="H1" s="3" t="s">
         <v>114</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="I1" s="3" t="s">
         <v>115</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>116</v>
       </c>
       <c r="J1" s="3" t="s">
         <v>46</v>
@@ -2920,10 +2889,10 @@
         <v>47</v>
       </c>
       <c r="L1" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="M1" s="3" t="s">
         <v>117</v>
-      </c>
-      <c r="M1" s="3" t="s">
-        <v>118</v>
       </c>
       <c r="N1" s="3" t="s">
         <v>48</v>
@@ -2932,7 +2901,7 @@
         <v>49</v>
       </c>
       <c r="P1" s="3" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="Q1" s="3" t="s">
         <v>71</v>
@@ -2975,19 +2944,19 @@
         <v>66</v>
       </c>
       <c r="C1" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>108</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>109</v>
       </c>
     </row>
   </sheetData>
@@ -3015,7 +2984,7 @@
         <v>66</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
   </sheetData>
@@ -3045,10 +3014,10 @@
         <v>66</v>
       </c>
       <c r="C1" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>102</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>103</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>37</v>
@@ -3082,10 +3051,10 @@
         <v>66</v>
       </c>
       <c r="C1" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>102</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>103</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>37</v>
@@ -3119,10 +3088,10 @@
         <v>66</v>
       </c>
       <c r="C1" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>102</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>103</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>37</v>
@@ -3136,7 +3105,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:K1"/>
+  <dimension ref="A1:J1"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22.44140625" style="1" bestFit="1" customWidth="1"/>
@@ -3146,13 +3115,12 @@
     <col min="5" max="6" width="19.33203125" style="1" customWidth="1"/>
     <col min="7" max="7" width="9" style="1" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="9" style="1" customWidth="1"/>
-    <col min="9" max="9" width="8.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="14.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="20.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="16384" width="9.109375" style="1"/>
+    <col min="9" max="9" width="14.5546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="20.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="16384" width="9.109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="2" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" s="2" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>52</v>
       </c>
@@ -3178,12 +3146,9 @@
         <v>3</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>94</v>
+        <v>75</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="K1" s="2" t="s">
         <v>20</v>
       </c>
     </row>
@@ -3223,13 +3188,13 @@
   <sheetData>
     <row r="1" spans="1:19" s="2" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="C1" s="2" t="s">
         <v>97</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>98</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>52</v>
@@ -3250,7 +3215,7 @@
         <v>23</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="K1" s="2" t="s">
         <v>24</v>
@@ -3309,13 +3274,13 @@
   <sheetData>
     <row r="1" spans="1:13" s="2" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>97</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>98</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>52</v>
@@ -3324,10 +3289,10 @@
         <v>66</v>
       </c>
       <c r="F1" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="G1" s="2" t="s">
         <v>100</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>101</v>
       </c>
       <c r="H1" s="2" t="s">
         <v>4</v>
@@ -3376,22 +3341,22 @@
   <sheetData>
     <row r="1" spans="1:12" s="2" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>136</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>137</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>36</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>89</v>
@@ -3437,22 +3402,22 @@
   <sheetData>
     <row r="1" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>136</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>137</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>36</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>88</v>
@@ -3495,19 +3460,19 @@
   <sheetData>
     <row r="1" spans="1:11" s="2" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="B1" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>137</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>138</v>
       </c>
       <c r="F1" s="2" t="s">
         <v>89</v>
@@ -3554,25 +3519,25 @@
   <sheetData>
     <row r="1" spans="1:11" s="2" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>97</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>98</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>38</v>
       </c>
       <c r="E1" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="F1" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>134</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>135</v>
       </c>
       <c r="H1" s="2" t="s">
         <v>39</v>
@@ -3614,16 +3579,16 @@
   <sheetData>
     <row r="1" spans="1:10" s="2" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>127</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>128</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>11</v>
@@ -3635,13 +3600,13 @@
         <v>66</v>
       </c>
       <c r="H1" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="I1" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>130</v>
-      </c>
-      <c r="J1" s="2" t="s">
-        <v>131</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix(fix-B-024): adjust on new position history echelons list
</commit_message>
<xml_diff>
--- a/public/template_excel/DATA PEGAWAI ASN.xlsx
+++ b/public/template_excel/DATA PEGAWAI ASN.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27928"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\api\public\template_excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\simdatuk-dev\public\template_excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E86E771C-D997-49DF-B8F7-4D80652BB313}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="23260" windowHeight="12460" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Data Pegawai" sheetId="1" r:id="rId1"/>
@@ -41,12 +40,12 @@
 </file>
 
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Windows User</author>
   </authors>
   <commentList>
-    <comment ref="H1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000001000000}">
+    <comment ref="H1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -75,7 +74,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="I1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000002000000}">
+    <comment ref="I1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -100,7 +99,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000003000000}">
+    <comment ref="J1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -128,7 +127,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="M1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000004000000}">
+    <comment ref="M1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -155,7 +154,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="P1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000005000000}">
+    <comment ref="P1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -185,7 +184,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="R1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000006000000}">
+    <comment ref="R1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -243,7 +242,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="T1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000007000000}">
+    <comment ref="T1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -280,7 +279,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="V1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000008000000}">
+    <comment ref="V1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -330,7 +329,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="W1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000009000000}">
+    <comment ref="W1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -361,7 +360,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AG1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000A000000}">
+    <comment ref="AG1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -393,7 +392,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AJ1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000B000000}">
+    <comment ref="AJ1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -431,12 +430,12 @@
 </file>
 
 <file path=xl/comments10.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Windows User</author>
   </authors>
   <commentList>
-    <comment ref="B1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0900-000001000000}">
+    <comment ref="B1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -471,7 +470,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="H1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0900-000002000000}">
+    <comment ref="H1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -504,12 +503,12 @@
 </file>
 
 <file path=xl/comments11.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Windows User</author>
   </authors>
   <commentList>
-    <comment ref="B1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0A00-000001000000}">
+    <comment ref="B1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -544,7 +543,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="H1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0A00-000002000000}">
+    <comment ref="H1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -583,12 +582,12 @@
 </file>
 
 <file path=xl/comments12.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Windows User</author>
   </authors>
   <commentList>
-    <comment ref="F1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0B00-000001000000}">
+    <comment ref="F1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -613,7 +612,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="G1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0B00-000002000000}">
+    <comment ref="G1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -642,7 +641,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="L1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0B00-000003000000}">
+    <comment ref="L1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -676,7 +675,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="M1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0B00-000004000000}">
+    <comment ref="M1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -709,7 +708,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="P1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0B00-000005000000}">
+    <comment ref="P1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -741,12 +740,12 @@
 </file>
 
 <file path=xl/comments13.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Windows User</author>
   </authors>
   <commentList>
-    <comment ref="E1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0C00-000001000000}">
+    <comment ref="E1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -780,12 +779,12 @@
 </file>
 
 <file path=xl/comments14.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Windows User</author>
   </authors>
   <commentList>
-    <comment ref="D1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0E00-000001000000}">
+    <comment ref="D1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -816,12 +815,12 @@
 </file>
 
 <file path=xl/comments15.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Windows User</author>
   </authors>
   <commentList>
-    <comment ref="D1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0F00-000001000000}">
+    <comment ref="D1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -851,12 +850,12 @@
 </file>
 
 <file path=xl/comments16.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Windows User</author>
   </authors>
   <commentList>
-    <comment ref="D1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-1000-000001000000}">
+    <comment ref="D1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -893,12 +892,12 @@
 </file>
 
 <file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Windows User</author>
   </authors>
   <commentList>
-    <comment ref="C1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000001000000}">
+    <comment ref="C1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -929,7 +928,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000002000000}">
+    <comment ref="E1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -959,12 +958,12 @@
 </file>
 
 <file path=xl/comments3.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Windows User</author>
   </authors>
   <commentList>
-    <comment ref="B1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000001000000}">
+    <comment ref="B1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -999,7 +998,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="H1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000002000000}">
+    <comment ref="H1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -1022,13 +1021,14 @@
 - Eselon I
 - Eselon II
 - Eselon III
+- Eselon IV
+- Pelaksana
 - Fungsional
-- Pelaksana
 - Staf</t>
         </r>
       </text>
     </comment>
-    <comment ref="I1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000003000000}">
+    <comment ref="I1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -1060,12 +1060,12 @@
 </file>
 
 <file path=xl/comments4.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Windows User</author>
   </authors>
   <commentList>
-    <comment ref="B1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0300-000001000000}">
+    <comment ref="B1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -1100,7 +1100,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="F1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0300-000002000000}">
+    <comment ref="F1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -1157,7 +1157,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="I1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0300-000003000000}">
+    <comment ref="I1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -1196,7 +1196,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="M1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0300-000004000000}">
+    <comment ref="M1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -1226,12 +1226,12 @@
 </file>
 
 <file path=xl/comments5.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Windows User</author>
   </authors>
   <commentList>
-    <comment ref="B1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0400-000001000000}">
+    <comment ref="B1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -1266,7 +1266,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0400-000002000000}">
+    <comment ref="E1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -1300,12 +1300,12 @@
 </file>
 
 <file path=xl/comments6.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Windows User</author>
   </authors>
   <commentList>
-    <comment ref="B1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0500-000001000000}">
+    <comment ref="B1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -1340,7 +1340,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0500-000002000000}">
+    <comment ref="E1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -1375,12 +1375,12 @@
 </file>
 
 <file path=xl/comments7.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Windows User</author>
   </authors>
   <commentList>
-    <comment ref="B1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0600-000001000000}">
+    <comment ref="B1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -1415,7 +1415,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="I1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0600-000002000000}">
+    <comment ref="I1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -1475,12 +1475,12 @@
 </file>
 
 <file path=xl/comments8.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Windows User</author>
   </authors>
   <commentList>
-    <comment ref="A1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0700-000001000000}">
+    <comment ref="A1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -1509,7 +1509,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0700-000002000000}">
+    <comment ref="B1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -1544,7 +1544,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0700-000003000000}">
+    <comment ref="E1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -1588,12 +1588,12 @@
 </file>
 
 <file path=xl/comments9.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Windows User</author>
   </authors>
   <commentList>
-    <comment ref="B1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0800-000001000000}">
+    <comment ref="B1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -1628,7 +1628,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0800-000002000000}">
+    <comment ref="D1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -1656,7 +1656,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="H1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0800-000003000000}">
+    <comment ref="H1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -1682,7 +1682,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="I1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0800-000004000000}">
+    <comment ref="I1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -1710,7 +1710,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0800-000005000000}">
+    <comment ref="J1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -2160,7 +2160,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -2510,57 +2510,57 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:AS3"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.08984375" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="22.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="22.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="22.453125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.54296875" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.36328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.54296875" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="22.36328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.6328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.90625" style="1" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="12" style="1" customWidth="1"/>
-    <col min="9" max="9" width="15.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="21.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="20.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="24.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="19.33203125" style="1" customWidth="1"/>
-    <col min="14" max="14" width="21.5546875" style="1" customWidth="1"/>
-    <col min="15" max="15" width="17.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="84.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="17.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="33.109375" style="1" customWidth="1"/>
-    <col min="19" max="19" width="30.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.90625" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="21.453125" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="20.6328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="24.90625" style="1" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="19.36328125" style="1" customWidth="1"/>
+    <col min="14" max="14" width="21.54296875" style="1" customWidth="1"/>
+    <col min="15" max="15" width="17.36328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="84.453125" style="1" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="17.36328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="33.08984375" style="1" customWidth="1"/>
+    <col min="19" max="19" width="30.453125" style="1" bestFit="1" customWidth="1"/>
     <col min="20" max="21" width="29" style="1" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="28.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="27.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="27.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="31.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="31.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="28.36328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="27.453125" style="1" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="27.36328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="31.90625" style="1" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="31.36328125" style="1" bestFit="1" customWidth="1"/>
     <col min="27" max="27" width="29" style="1" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="39.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="58.33203125" style="1" customWidth="1"/>
-    <col min="30" max="30" width="36.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="36.109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="17.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="39.54296875" style="1" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="58.36328125" style="1" customWidth="1"/>
+    <col min="30" max="30" width="36.6328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="36.08984375" style="1" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="17.36328125" style="1" bestFit="1" customWidth="1"/>
     <col min="33" max="33" width="23" style="1" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="19.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="35" max="36" width="25.33203125" style="1" customWidth="1"/>
-    <col min="37" max="37" width="73.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="27.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="19.90625" style="1" bestFit="1" customWidth="1"/>
+    <col min="35" max="36" width="25.36328125" style="1" customWidth="1"/>
+    <col min="37" max="37" width="73.90625" style="1" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="27.90625" style="1" bestFit="1" customWidth="1"/>
     <col min="39" max="39" width="20" style="1" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="13.109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="15.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="19.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="16.109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="44" max="44" width="15.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="45" max="45" width="73.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="46" max="16384" width="9.109375" style="1"/>
+    <col min="40" max="40" width="13.08984375" style="1" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="15.453125" style="1" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="19.90625" style="1" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="16.08984375" style="1" bestFit="1" customWidth="1"/>
+    <col min="44" max="44" width="15.36328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="73.90625" style="1" bestFit="1" customWidth="1"/>
+    <col min="46" max="16384" width="9.08984375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:45" s="2" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:45" s="2" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>53</v>
       </c>
@@ -2697,7 +2697,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="3" spans="1:45" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="3" spans="1:45" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -2706,22 +2706,22 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H1"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.08984375" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="24.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="31.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="24.6328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="31.453125" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="32" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="24.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="24.6640625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="21.109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="18.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="16384" width="9.109375" style="1"/>
+    <col min="4" max="4" width="18.90625" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="24.6328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="24.6328125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="21.08984375" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.90625" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="16384" width="9.08984375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="2" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" s="2" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>123</v>
       </c>
@@ -2754,28 +2754,28 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:O1"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.08984375" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="35.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="31.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="35.453125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="31.453125" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="32" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17.33203125" style="1" customWidth="1"/>
-    <col min="6" max="6" width="22.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="26.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="25.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.36328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.36328125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="22.6328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.54296875" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="26.90625" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="25.6328125" style="1" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="30" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="34.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="34.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="13" max="14" width="26.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="16" max="16384" width="9.109375" style="1"/>
+    <col min="11" max="11" width="34.36328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="34.6328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="13" max="14" width="26.90625" style="1" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.36328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="16" max="16384" width="9.08984375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:15" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>119</v>
       </c>
@@ -2829,32 +2829,32 @@
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:S1"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.08984375" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="22.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.44140625" style="1" customWidth="1"/>
+    <col min="1" max="1" width="22.453125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.453125" style="1" customWidth="1"/>
     <col min="3" max="3" width="21" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="27" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="22.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.36328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.90625" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.453125" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.6328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.90625" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.453125" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10.453125" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="22.453125" style="1" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="25" style="1" bestFit="1" customWidth="1"/>
-    <col min="14" max="15" width="24.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="21.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="21.44140625" style="1" customWidth="1"/>
-    <col min="18" max="18" width="13.109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="14.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="20" max="16384" width="9.109375" style="1"/>
+    <col min="14" max="15" width="24.90625" style="1" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="21.453125" style="1" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="21.453125" style="1" customWidth="1"/>
+    <col min="18" max="18" width="13.08984375" style="1" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="14.6328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="20" max="16384" width="9.08984375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" s="3" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:19" s="3" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>52</v>
       </c>
@@ -2921,22 +2921,22 @@
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:G1"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.08984375" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="22.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.44140625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="21.109375" style="1" customWidth="1"/>
-    <col min="4" max="4" width="21.6640625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="29.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.109375" style="1" customWidth="1"/>
-    <col min="7" max="7" width="16.33203125" style="1" customWidth="1"/>
-    <col min="8" max="8" width="10.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="16384" width="9.109375" style="1"/>
+    <col min="1" max="1" width="22.453125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.453125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="21.08984375" style="1" customWidth="1"/>
+    <col min="4" max="4" width="21.6328125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="29.6328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.08984375" style="1" customWidth="1"/>
+    <col min="7" max="7" width="16.36328125" style="1" customWidth="1"/>
+    <col min="8" max="8" width="10.6328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="16384" width="9.08984375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="2" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" s="2" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>52</v>
       </c>
@@ -2966,17 +2966,17 @@
 </file>
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0D00-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:C1"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.08984375" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="22.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.44140625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="23.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="16384" width="9.109375" style="1"/>
+    <col min="1" max="1" width="22.453125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.453125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="23.54296875" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="16384" width="9.08984375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="2" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" s="2" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>52</v>
       </c>
@@ -2993,20 +2993,20 @@
 </file>
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0E00-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:E1"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.08984375" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="22.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.44140625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="10.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="22.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="22.453125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.453125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="10.6328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22.6328125" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="18" style="1" customWidth="1"/>
-    <col min="6" max="6" width="16.109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="16384" width="9.109375" style="1"/>
+    <col min="6" max="6" width="16.08984375" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="16384" width="9.08984375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="2" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" s="2" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>52</v>
       </c>
@@ -3030,20 +3030,20 @@
 </file>
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0F00-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:E1"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.08984375" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="22.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.44140625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="10.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.33203125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="15.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="16384" width="9.109375" style="1"/>
+    <col min="1" max="1" width="22.453125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.453125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="10.6328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.36328125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="15.54296875" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.08984375" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="16384" width="9.08984375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="2" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" s="2" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>52</v>
       </c>
@@ -3067,20 +3067,20 @@
 </file>
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:E1"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.08984375" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="22.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.44140625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="10.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="22.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18.33203125" style="1" customWidth="1"/>
-    <col min="6" max="6" width="16.109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="16384" width="9.109375" style="1"/>
+    <col min="1" max="1" width="22.453125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.453125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="10.6328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22.6328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.36328125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="16.08984375" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="16384" width="9.08984375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="2" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" s="2" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>52</v>
       </c>
@@ -3104,23 +3104,23 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:J1"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.08984375" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="22.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.44140625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="22.5546875" style="1" customWidth="1"/>
-    <col min="4" max="4" width="19.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="19.33203125" style="1" customWidth="1"/>
+    <col min="1" max="1" width="22.453125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.453125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="22.54296875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="19.36328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="19.36328125" style="1" customWidth="1"/>
     <col min="7" max="7" width="9" style="1" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="9" style="1" customWidth="1"/>
-    <col min="9" max="9" width="14.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="20.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="16384" width="9.109375" style="1"/>
+    <col min="9" max="9" width="14.54296875" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="20.90625" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="16384" width="9.08984375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="2" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" s="2" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>52</v>
       </c>
@@ -3160,33 +3160,33 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:S1"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.08984375" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="31.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="31.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="31.54296875" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="31.453125" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="32" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="22.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="22.44140625" style="1" customWidth="1"/>
-    <col min="6" max="6" width="31.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="24.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="16.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="20.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22.453125" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="22.453125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="31.54296875" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="24.6328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.54296875" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="20.6328125" style="1" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="20" style="1" customWidth="1"/>
-    <col min="11" max="11" width="11.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="16.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="15.109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.54296875" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="16.90625" style="1" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="15.08984375" style="1" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="20" style="1" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="16.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="16.6328125" style="1" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="19" style="1" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="34.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="27.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="24.109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="20" max="16384" width="9.109375" style="1"/>
+    <col min="17" max="17" width="34.90625" style="1" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="27.36328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="24.08984375" style="1" bestFit="1" customWidth="1"/>
+    <col min="20" max="16384" width="9.08984375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" s="2" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:19" s="2" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>95</v>
       </c>
@@ -3252,27 +3252,27 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:M1"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.08984375" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="32.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="31.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="32.453125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="31.453125" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="32" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17.33203125" style="1" customWidth="1"/>
-    <col min="6" max="6" width="18.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="17.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.36328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.36328125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="18.90625" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.6328125" style="1" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="22" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="22.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="22.6328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.453125" style="1" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="22" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="22.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="17.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="14" max="16384" width="9.109375" style="1"/>
+    <col min="12" max="12" width="22.6328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="17.453125" style="1" bestFit="1" customWidth="1"/>
+    <col min="14" max="16384" width="9.08984375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" s="2" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" s="2" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>98</v>
       </c>
@@ -3321,25 +3321,25 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:L1"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.08984375" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="26" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="31.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="31.453125" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="32" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="22.109375" style="1" customWidth="1"/>
-    <col min="6" max="6" width="23.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.6328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="22.08984375" style="1" customWidth="1"/>
+    <col min="6" max="6" width="23.453125" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="29" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="23.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="15.5546875" style="1" customWidth="1"/>
-    <col min="11" max="11" width="17.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="16384" width="9.109375" style="1"/>
+    <col min="8" max="8" width="23.453125" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.54296875" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.54296875" style="1" customWidth="1"/>
+    <col min="11" max="11" width="17.36328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="16384" width="9.08984375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" s="2" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" s="2" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>135</v>
       </c>
@@ -3384,23 +3384,23 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:K1"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.08984375" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="53.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="31.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="53.6328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="31.453125" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="32" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="23.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.6328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="23.453125" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="29" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="23.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="16384" width="9.109375" style="1"/>
+    <col min="8" max="8" width="23.453125" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.54296875" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.36328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="16384" width="9.08984375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>135</v>
       </c>
@@ -3443,22 +3443,22 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:K1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="14.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="31.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.90625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="31.453125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="32" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="23.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.6328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="23.453125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.5546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.5546875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15.5546875" customWidth="1"/>
+    <col min="7" max="7" width="14.54296875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.54296875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="2" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" s="2" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>135</v>
       </c>
@@ -3500,24 +3500,24 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:K1"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.08984375" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="22.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="31.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="22.453125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="31.453125" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="32" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="52.109375" style="1" customWidth="1"/>
-    <col min="5" max="5" width="34.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="22.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="52.08984375" style="1" customWidth="1"/>
+    <col min="5" max="5" width="34.90625" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.453125" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="22.453125" style="1" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="16" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="31.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="16384" width="9.109375" style="1"/>
+    <col min="9" max="9" width="31.36328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.36328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="16384" width="9.08984375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="2" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" s="2" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>131</v>
       </c>
@@ -3560,24 +3560,24 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:J1"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.08984375" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="27.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="31.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="27.6328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="31.453125" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="32" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="26" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.88671875" style="1" customWidth="1"/>
-    <col min="6" max="6" width="17.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="17.33203125" style="1" customWidth="1"/>
-    <col min="8" max="8" width="23.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="27.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.90625" style="1" customWidth="1"/>
+    <col min="6" max="6" width="17.36328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.36328125" style="1" customWidth="1"/>
+    <col min="8" max="8" width="23.54296875" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="27.6328125" style="1" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="29" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="16384" width="9.109375" style="1"/>
+    <col min="11" max="16384" width="9.08984375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="2" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" s="2" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>126</v>
       </c>

</xml_diff>

<commit_message>
chore: change TMT Menjabat to TMT Jabatan
</commit_message>
<xml_diff>
--- a/public/template_excel/DATA PEGAWAI ASN.xlsx
+++ b/public/template_excel/DATA PEGAWAI ASN.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="23260" windowHeight="12460" activeTab="2"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="23260" windowHeight="12460"/>
   </bookViews>
   <sheets>
     <sheet name="Data Pegawai" sheetId="1" r:id="rId1"/>
@@ -2025,9 +2025,6 @@
     <t xml:space="preserve">Nama Sekolah </t>
   </si>
   <si>
-    <t xml:space="preserve">TMT Menjabat </t>
-  </si>
-  <si>
     <t xml:space="preserve">Nama Riwayat Jabatan </t>
   </si>
   <si>
@@ -2155,6 +2152,9 @@
   </si>
   <si>
     <t xml:space="preserve">Tanggal Pelaksanaan </t>
+  </si>
+  <si>
+    <t>TMT Jabatan</t>
   </si>
 </sst>
 </file>
@@ -2723,16 +2723,16 @@
   <sheetData>
     <row r="1" spans="1:8" s="2" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>123</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>124</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>52</v>
@@ -2741,7 +2741,7 @@
         <v>66</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="H1" s="2" t="s">
         <v>41</v>
@@ -2777,13 +2777,13 @@
   <sheetData>
     <row r="1" spans="1:15" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>96</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>97</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>52</v>
@@ -2798,7 +2798,7 @@
         <v>9</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="I1" s="2" t="s">
         <v>42</v>
@@ -2807,10 +2807,10 @@
         <v>43</v>
       </c>
       <c r="K1" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="L1" s="2" t="s">
         <v>121</v>
-      </c>
-      <c r="L1" s="2" t="s">
-        <v>122</v>
       </c>
       <c r="M1" s="2" t="s">
         <v>44</v>
@@ -2862,25 +2862,25 @@
         <v>66</v>
       </c>
       <c r="C1" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="D1" s="3" t="s">
         <v>109</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="E1" s="3" t="s">
         <v>110</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="F1" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="G1" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="H1" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="I1" s="3" t="s">
         <v>114</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>115</v>
       </c>
       <c r="J1" s="3" t="s">
         <v>46</v>
@@ -2889,10 +2889,10 @@
         <v>47</v>
       </c>
       <c r="L1" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="M1" s="3" t="s">
         <v>116</v>
-      </c>
-      <c r="M1" s="3" t="s">
-        <v>117</v>
       </c>
       <c r="N1" s="3" t="s">
         <v>48</v>
@@ -2901,7 +2901,7 @@
         <v>49</v>
       </c>
       <c r="P1" s="3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="Q1" s="3" t="s">
         <v>71</v>
@@ -2944,19 +2944,19 @@
         <v>66</v>
       </c>
       <c r="C1" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>107</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>108</v>
       </c>
     </row>
   </sheetData>
@@ -2984,7 +2984,7 @@
         <v>66</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
   </sheetData>
@@ -3014,10 +3014,10 @@
         <v>66</v>
       </c>
       <c r="C1" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>101</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>102</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>37</v>
@@ -3051,10 +3051,10 @@
         <v>66</v>
       </c>
       <c r="C1" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>101</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>102</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>37</v>
@@ -3088,10 +3088,10 @@
         <v>66</v>
       </c>
       <c r="C1" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>101</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>102</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>37</v>
@@ -3188,13 +3188,13 @@
   <sheetData>
     <row r="1" spans="1:19" s="2" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="C1" s="2" t="s">
         <v>96</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>97</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>52</v>
@@ -3215,7 +3215,7 @@
         <v>23</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>94</v>
+        <v>137</v>
       </c>
       <c r="K1" s="2" t="s">
         <v>24</v>
@@ -3274,13 +3274,13 @@
   <sheetData>
     <row r="1" spans="1:13" s="2" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>96</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>97</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>52</v>
@@ -3289,10 +3289,10 @@
         <v>66</v>
       </c>
       <c r="F1" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="G1" s="2" t="s">
         <v>99</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>100</v>
       </c>
       <c r="H1" s="2" t="s">
         <v>4</v>
@@ -3341,22 +3341,22 @@
   <sheetData>
     <row r="1" spans="1:12" s="2" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>135</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>136</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>36</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>89</v>
@@ -3402,22 +3402,22 @@
   <sheetData>
     <row r="1" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>135</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>136</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>36</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>88</v>
@@ -3460,19 +3460,19 @@
   <sheetData>
     <row r="1" spans="1:11" s="2" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="B1" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>136</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>137</v>
       </c>
       <c r="F1" s="2" t="s">
         <v>89</v>
@@ -3519,25 +3519,25 @@
   <sheetData>
     <row r="1" spans="1:11" s="2" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>96</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>97</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>38</v>
       </c>
       <c r="E1" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="F1" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>133</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>134</v>
       </c>
       <c r="H1" s="2" t="s">
         <v>39</v>
@@ -3579,16 +3579,16 @@
   <sheetData>
     <row r="1" spans="1:10" s="2" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>126</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>127</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>11</v>
@@ -3600,13 +3600,13 @@
         <v>66</v>
       </c>
       <c r="H1" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="I1" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>129</v>
-      </c>
-      <c r="J1" s="2" t="s">
-        <v>130</v>
       </c>
     </row>
   </sheetData>

</xml_diff>